<commit_message>
update main with dictionary-based NER model only
</commit_message>
<xml_diff>
--- a/ds-lab2/annotated_skill_roles.xlsx
+++ b/ds-lab2/annotated_skill_roles.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:M13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -481,10 +481,15 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
+          <t>annotated_key_knowledge</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
           <t>unique_task_phrases</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>unique_skill_phrases</t>
         </is>
@@ -501,10 +506,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Defines, maintains and communicates the cybersecurity vision, strategy, policies and
-procedures. Manages the implementation of the cybersecurity policy across the
-organisation. Assures information exchange with external authorities and professional
-bodies.</t>
+          <t>Defines maintains and communicates the cybersecurity vision strategy policies and procedures. Manages the implementation of the cybersecurity policy across the organisation. Assures information exchange with external authorities and professional bodies.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -515,85 +517,47 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Define, implement, communicate and maintain cybersecurity goals, requirements,
-strategies, policies, aligned with the business strategy to support the organisational
-objectives
- Prepare and present cybersecurity vision, strategies and policies for approval by the
-senior management of the organisation and ensure their execution
- Supervise the application and improvement of the Information Security Management
-System (ISMS)
- Educate senior management about cybersecurity risks, threats and their impact to
-the organisation
- Ensure the senior management approves the cybersecurity risks of the organisation
- Develop cybersecurity plans
- Develop relationships with cybersecurity-related authorities and communities
- Report cybersecurity incidents, risks, findings to the senior management
- Monitor advancement in cybersecurity
- Secure resources to implement the cybersecurity strategy
- Negotiate the cybersecurity budget with the senior management
- Ensure the organisation’s resiliency to cyber incidents
- Manage continuous capacity building within the organisation
- Review, plan and allocate appropriate cybersecurity resources</t>
+          <t>Define implement communicate and maintain cybersecurity goals requirements strategies policies aligned with the business strategy to support the organisational objectives Prepare and present cybersecurity vision strategies and policies for approval by the senior management of the organisation and ensure their execution Supervise the application and improvement of the Information Security Management System (ISMS) Educate senior management about cybersecurity risks threats and their impact to the organisation Ensure the senior management approves the cybersecurity risks of the organisation Develop cybersecurity plans Develop relationships with cybersecurity-related authorities and communities Report cybersecurity incidents risks findings to the senior management Monitor advancement in cybersecurity Secure resources to implement the cybersecurity strategy Negotiate the cybersecurity budget with the senior management Ensure the organisation’s resiliency to cyber incidents Manage continuous capacity building within the organisation Review plan and allocate appropriate cybersecurity resources</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Assess and enhance an organisation’s cybersecurity posture  Analyse and implement cybersecurity policies, certifications, standards, methodologies and frameworks  Analyse and comply with cybersecurity-related laws, regulations and legislations  Implement cybersecurity recommendations and best practices  Manage cybersecurity resources  Develop, champion and lead the execution of a cybersecurity strategy  Influence an organisation’s cybersecurity culture  Design, apply, monitor and review Information Security Management System (ISMS) either directly or by leading its outsourcing  Review and enhance security documents, reports, SLAs and ensure the security objectives  Identify and solve cybersecurity-related issues  Establish a cybersecurity plan  Communicate, coordinate and cooperate with internal and external stakeholders  Anticipate required changes to the organisation’s information security strategy and formulate new plans  Define and apply maturity models for cybersecurity management
- Anticipate cybersecurity threats, needs and upcoming challenges
- Motivate and encourage people</t>
+          <t>Assess and enhance an organisation’s cybersecurity posture Analyse and implement cybersecurity policies certifications standards methodologies and frameworks Analyse and comply with cybersecurity-related laws regulations and legislations Implement cybersecurity recommendations and best practices Manage cybersecurity resources Develop champion and lead the execution of a cybersecurity strategy Influence an organisation’s cybersecurity culture Design apply monitor and review Information Security Management System (ISMS) either directly or by leading its outsourcing Review and enhance security documents reports SLAs and ensure the security objectives Identify and solve cybersecurity-related issues Establish a cybersecurity plan Communicate coordinate and cooperate with internal and external stakeholders Anticipate required changes to the organisation’s information security strategy and formulate new plans Define and apply maturity models for cybersecurity management Anticipate cybersecurity threats needs and upcoming challenges Motivate and encourage people</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Cybersecurity policies  Cybersecurity standards, methodologies and frameworks  Cybersecurity recommendations and best practices  Cybersecurity related laws, regulations and legislations  Cybersecurity-related certifications  Ethical cybersecurity organisation requirements  Cybersecurity maturity models  Cybersecurity procedures  Resource management  Management practices  Risk management standards, methodologies and frameworks</t>
+          <t>Cybersecurity policies Cybersecurity standards methodologies and frameworks Cybersecurity recommendations and best practices Cybersecurity related laws regulations and legislations Cybersecurity-related certifications Ethical cybersecurity organisation requirements Cybersecurity maturity models Cybersecurity procedures Resource management Management practices Risk management standards methodologies and frameworks</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Defines, maintains and communicates the [cybersecurity](SKILLS) vision, strategy, policies and
-procedures. Manages the [implementation](SKILLS) of the [cybersecurity](SKILLS) policy across the
-organisation. Assures information exchange with external authorities and professional
-bodies.</t>
+          <t>[Defines](TASK) [maintains](TASK) and [communicates](TASK) the [cybersecurity](SKILLS) vision [strategy policies](SKILLS) and procedures. [Manages](TASK) the [implementation](SKILLS) of the [cybersecurity](SKILLS) [policy](SKILLS) across the organisation. Assures information exchange with external authorities and professional bodies.</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> [Define](TASK), [implement](TASK), [communicate](TASK) and [maintain](TASK) [cybersecurity](SKILLS) goals, requirements,
-strategies, policies, aligned with the [business strategy](SKILLS) to [support[](TASK)](SKILLS) the organisational
-objectives
- [Prepare](TASK) and [present](TASK) [cybersecurity](SKILLS) vision, strategies and policies for approval by the
-senior management of the organisation and [ensure](TASK) their execution
- [Supervise](TASK) the application and improvement of the Information Security Management
-System (ISMS)
- [Educate](TASK) senior management about [cybersecurity](SKILLS) risks, threats and their impact to
-the organisation
- [Ensure](TASK) the senior management approves the [cybersecurity](SKILLS) risks of the organisation
- [Develop](TASK) [cybersecurity](SKILLS) plans
- [Develop](TASK) relationships with [cybersecurity](SKILLS)-related authorities and communities
- [Report](TASK) [cybersecurity](SKILLS) incidents, risks, findings to the senior management
- [Monitor](TASK) advancement in [cybersecurity](SKILLS)
- [Secure](TASK) resources to [implement](TASK) the [cybersecurity](SKILLS) strategy
- [Negotiate](TASK) the [cybersecurity](SKILLS) budget with the senior management
- [Ensure](TASK) the organisation’s resiliency to cyber incidents
- [Manage](TASK) continuous capacity building within the organisation
- [Review](TASK), plan and [allocate](TASK) appropriate [cybersecurity](SKILLS) resources</t>
+          <t>[Define](TASK) [implement](TASK) [communicate](TASK) and [maintain](TASK) [cybersecurity](SKILLS) goals requirements [strategies policies](SKILLS) aligned with the [business strategy](SKILLS) to [support](TASK) the organisational objectives Prepare and [present](TASK) [cybersecurity](SKILLS) vision [strategies](SKILLS) and [policies](SKILLS) for approval by the senior management of the organisation and [ensure](TASK) their execution [Supervise](TASK) the application and improvement of the [Information Security Management System](SKILLS) (ISMS) [Educate](TASK) senior management about [cybersecurity risks](SKILLS) threats and their impact to the organisation [Ensure](TASK) the senior management approves the [cybersecurity risks](SKILLS) of the organisation [Develop](TASK) [cybersecurity](SKILLS) plans [Develop](TASK) relationships with [cybersecurity](SKILLS)-related authorities and communities [Report](TASK) [cybersecurity incidents](SKILLS) risks findings to the senior management [Monitor](TASK) advancement in [cybersecurity](SKILLS) [Secure][(TASK) resources](SKILLS) to [implement](TASK) the [cybersecurity strategy](SKILLS) [Negotiate](TASK) the [cybersecurity](SKILLS) budget with the senior management [Ensure](TASK) the organisation’s resiliency to [cyber](SKILLS) incidents [Manage](TASK) continuous capacity building within the organisation [Review](TASK) plan and [allocate](TASK) appropriate [cybersecurity resources](SKILLS)</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>[Assess](TASK) and [enhance](TASK) an organisation’s [cybersecurity](SKILLS) posture  [Analyse](TASK) and [implement](TASK) [cybersecurity](SKILLS) policies, [certifications](SKILLS), standards, [methodologies](SKILLS) and [frameworks](SKILLS)  [Analyse](TASK) and comply with [cybersecurity](SKILLS)-related laws, regulations and legislations  [Implement](TASK) [cybersecurity](SKILLS) [recommendations](SKILLS) and [best practices](SKILLS)  [Manage](TASK) [cybersecurity](SKILLS) resources  [Develop](TASK), champion and [lead](TASK) the execution of a [cybersecurity](SKILLS) strategy  Influence an organisation’s [cybersecurity](SKILLS) culture  [Design](TASK), [apply](TASK), [monitor](TASK) and [review](TASK) [Information Security Management System](SKILLS) (ISMS) either directly or by leading its outsourcing  [Review](TASK) and [enhance](TASK) [security documents](SKILLS), reports, SLAs and [ensure](TASK) the [security objectives](SKILLS)  [Identify](TASK) and [solve](TASK) [cybersecurity](SKILLS)-related issues  [Establish](TASK) a [cybersecurity](SKILLS) plan  [Communicate](TASK), [coordinate](TASK) and cooperate with internal and external [stakeholders](SKILLS)  [Anticipate](TASK) required changes to the organisation’s information security strategy and formulate new plans  [Define](TASK) and [apply](TASK) [maturity models for cybersecurity management](SKILLS)
- [Anticipate](TASK) [cybersecurity](SKILLS) threats, needs and upcoming challenges
- [Motivate](TASK) and [encourage](TASK) people</t>
+          <t>[Assess](TASK) and [enhance](TASK) an organisation’s [cybersecurity](SKILLS) posture [Analyse](TASK) and [implement](TASK) [cybersecurity](SKILLS) [policies](SKILLS) [certifications](SKILLS) [standards methodologies](SKILLS) and [frameworks](SKILLS) [Analyse](TASK) and comply with [cybersecurity-related laws](SKILLS) regulations and legislations [Implement](TASK) [cybersecurity](SKILLS) [recommendations](SKILLS) and [best practices](SKILLS) [Manage](TASK) [cybersecurity resources](SKILLS) [Develop](TASK) champion and [lead](TASK) the execution of a [cybersecurity strategy](SKILLS) Influence an organisation’s [cybersecurity culture](SKILLS) [Design](TASK) [apply](TASK) [monitor](TASK) and [review](TASK) [Information Security Management System](SKILLS) (ISMS) either directly or by leading its outsourcing [Review](TASK) and [enhance](TASK) [security documents](SKILLS) reports SLAs and [ensure](TASK) the [security objectives](SKILLS) [Identify](TASK) and [solve](TASK) [cybersecurity-related issues](SKILLS) [Establish](TASK) a [cybersecurity plan](SKILLS) [Communicate](TASK) [coordinate](TASK) and [cooperate](TASK) with internal and external stakeholders [Anticipate](TASK) required changes to the organisation’s [information security](SKILLS) [strategy](SKILLS) and formulate new plans [Define](TASK) and [apply](TASK) [maturity models for cybersecurity management](SKILLS) [Anticipate](TASK) [cybersecurity threats](SKILLS) needs and upcoming challenges [Motivate](TASK) and [encourage](TASK) people</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>['Analyse', 'Anticipate', 'Assess', 'Communicate', 'Define', 'Design', 'Develop', 'Educate', 'Ensure', 'Establish', 'Identify', 'Implement', 'Manage', 'Monitor', 'Motivate', 'Negotiate', 'Prepare', 'Report', 'Review', 'Secure', 'Supervise', 'allocate', 'apply', 'communicate', 'coordinate', 'encourage', 'enhance', 'ensure', 'implement', 'lead', 'maintain', 'monitor', 'present', 'review', 'solve', 'support']</t>
+          <t>[Cybersecurity](SKILLS) [policies](SKILLS) [Cybersecurity standards methodologies](SKILLS) and [frameworks](SKILLS) [Cybersecurity](SKILLS) [recommendations](SKILLS) and [best practices](SKILLS) [Cybersecurity](SKILLS) related [laws regulations](SKILLS) and legislations [Cybersecurity](SKILLS)-related [certifications](SKILLS) Ethical [cybersecurity](SKILLS) organisation requirements [Cybersecurity](SKILLS) maturity models [Cybersecurity](SKILLS) procedures [Resource management](SKILLS) [Management practices](SKILLS) [Risk management](SKILLS) [standards methodologies](SKILLS) and [frameworks](SKILLS)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>['Information Security Management System', 'best practices', 'business strategy', 'certifications', 'cybersecurity', 'frameworks', 'implementation', 'maturity models for cybersecurity management', 'methodologies', 'recommendations', 'security documents', 'security objectives', 'stakeholders', 'support']</t>
+          <t>['Analyse', 'Anticipate', 'Assess', 'Communicate', 'Define', 'Defines', 'Design', 'Develop', 'Educate', 'Ensure', 'Establish', 'Identify', 'Implement', 'Manage', 'Manages', 'Monitor', 'Motivate', 'Negotiate', 'Report', 'Review', 'Secure', 'Supervise', 'allocate', 'apply', 'communicate', 'communicates', 'cooperate', 'coordinate', 'encourage', 'enhance', 'ensure', 'implement', 'lead', 'maintain', 'maintains', 'monitor', 'present', 'review', 'solve', 'support']</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>['Cybersecurity', 'Cybersecurity standards methodologies', 'Information Security Management System', 'Management practices', 'Resource management', 'Risk management', 'Secure resources', 'best practices', 'business strategy', 'certifications', 'cyber', 'cybersecurity', 'cybersecurity culture', 'cybersecurity incidents', 'cybersecurity plan', 'cybersecurity resources', 'cybersecurity risks', 'cybersecurity strategy', 'cybersecurity threats', 'cybersecurity-related issues', 'cybersecurity-related laws', 'frameworks', 'implementation', 'information security', 'laws regulations', 'maturity models for cybersecurity management', 'policies', 'policy', 'recommendations', 'security documents', 'security objectives', 'standards methodologies', 'strategies', 'strategies policies', 'strategy', 'strategy policies']</t>
         </is>
       </c>
     </row>
@@ -608,7 +572,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Monitors and assesses systems’ cybersecurity state. Analyses, evaluates and mitigates the impact of cybersecurity incidents. Identifies cyber incidents root causes and malicious actors. According to the organisation’s Incident Response Plan, restores systems’ and processes’ functionalities to an operational state, collecting evidences and documenting actions taken.</t>
+          <t>Monitors and assesses systems’ cybersecurity state. Analyses evaluates and mitigates the impact of cybersecurity incidents. Identifies cyber incidents root causes and malicious actors. According to the organisation’s Incident Response Plan restores systems’ and processes’ functionalities to an operational state collecting evidences and documenting actions taken.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -619,65 +583,47 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Cybersecurity policies  Cybersecurity standards, methodologies and frameworks  Cybersecurity recommendations and best practices  Cybersecurity related laws, regulations and legislations  Cybersecurity-related certifications  Ethical cybersecurity organisation requirements  Cybersecurity maturity models  Cybersecurity procedures  Resource management  Management practices  Risk management standards, methodologies and frameworks</t>
+          <t>Cybersecurity policies Cybersecurity standards methodologies and frameworks Cybersecurity recommendations and best practices Cybersecurity related laws regulations and legislations Cybersecurity-related certifications Ethical cybersecurity organisation requirements Cybersecurity maturity models Cybersecurity procedures Resource management Management practices Risk management standards methodologies and frameworks</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Practice all technical, functional and operational aspects of cybersecurity incident  handling and response 
- Collect, analyse and correlate cyber threat information originating from multiple  sources 
- Work on operating systems, servers, clouds and relevant infrastructures 
- Work under pressure 
- Communicate, present and report to relevant stakeholders 
- Manage and analyse log files</t>
+          <t>Practice all technical functional and operational aspects of cybersecurity incident handling and response Collect analyse and correlate cyber threat information originating from multiple sources Work on operating systems servers clouds and relevant infrastructures Work under pressure Communicate present and report to relevant stakeholders Manage and analyse log files</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Incident handling standards, methodologies and frameworks 
- Incident handling recommendations and best practices 
- Incident handling tools 
- Incident handling communication procedures 
- Operating systems security 
- Computer networks security 
- Cyber threats 
- Cybersecurity attack procedures 
- Computer systems vulnerabilities 
- Cybersecurity-related certifications 
- Cybersecurity related laws, regulations and legislations 
- Secure Operation Centres (SOCs) operation 
- Computer Security Incident Response Teams (CSIRTs) operation
-</t>
+          <t>Incident handling standards methodologies and frameworks Incident handling recommendations and best practices Incident handling tools Incident handling communication procedures Operating systems security Computer networks security Cyber threats Cybersecurity attack procedures Computer systems vulnerabilities Cybersecurity-related certifications Cybersecurity related laws regulations and legislations Secure Operation Centres (SOCs) operation Computer Security Incident Response Teams (CSIRTs) operation</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Monitors and assesses [systems](SKILLS)’ [cybersecurity](SKILLS) state. Analyses, evaluates and mitigates the impact of [cybersecurity](SKILLS) incidents. Identifies cyber incidents root causes and malicious actors. According to the organisation’s Incident Response Plan, restores [systems](SKILLS)’ and processes’ functionalities to an operational state, collecting evidences and documenting actions taken.</t>
+          <t>Monitors and assesses [systems](SKILLS)’ [cybersecurity](SKILLS) state. [Analyses](TASK) [evaluates](TASK) and mitigates the impact of [cybersecurity incidents](SKILLS). Identifies [cyber](SKILLS) incidents root causes and malicious actors. According to the organisation’s Incident [Response](TASK) Plan restores [systems](SKILLS)’ and [processes](TASK)’ functionalities to an [operational](SKILLS) state collecting evidences and documenting actions taken.</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> [Cybersecurity](SKILLS) policies  [Cybersecurity](SKILLS) standards, [methodologies](SKILLS) and [frameworks](SKILLS)  [Cybersecurity](SKILLS) [recommendations](SKILLS) and [best practices](SKILLS)  [Cybersecurity](SKILLS) related laws, regulations and legislations  [Cybersecurity](SKILLS)-related [certifications](SKILLS)  Ethical [cybersecurity](SKILLS) organisation requirements  [Cybersecurity](SKILLS) maturity models  [Cybersecurity](SKILLS) procedures  [Resource management](SKILLS)  [Management practices](SKILLS)  [Risk management](SKILLS) standards, [methodologies](SKILLS) and [frameworks](SKILLS)</t>
+          <t>[Cybersecurity](SKILLS) [policies](SKILLS) [Cybersecurity standards methodologies](SKILLS) and [frameworks](SKILLS) [Cybersecurity](SKILLS) [recommendations](SKILLS) and [best practices](SKILLS) [Cybersecurity](SKILLS) related [laws regulations](SKILLS) and legislations [Cybersecurity](SKILLS)-related [certifications](SKILLS) Ethical [cybersecurity](SKILLS) organisation requirements [Cybersecurity](SKILLS) maturity models [Cybersecurity](SKILLS) procedures [Resource management](SKILLS) [Management practices](SKILLS) [Risk management](SKILLS) [standards methodologies](SKILLS) and [frameworks](SKILLS)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> [Practice](TASK) all technical, functional and [operational aspects](SKILLS) of [cybersecurity](SKILLS) incident  handling and response 
- [Collect](TASK), [analyse](TASK) and [correlate](TASK) cyber threat information originating from multiple  sources 
- [Work](TASK) on [operating systems](SKILLS), [servers](SKILLS), [clouds](SKILLS) and relevant [infrastructures](SKILLS) 
- [Work](TASK) under pressure 
- [Communicate](TASK), [present](TASK) and [report](TASK) to relevant [stakeholders](SKILLS) 
- [Manage](TASK) and [analyse](TASK) [log files](SKILLS)</t>
+          <t>[Practice](TASK) all technical functional and [operational aspects](SKILLS) of [cybersecurity](SKILLS) incident handling and [response](TASK) Collect [analyse](TASK) and [correlate](TASK) [cyber threat](SKILLS) information originating from multiple sources [Work](TASK) on [operating systems](SKILLS) servers [clouds](SKILLS) and relevant infrastructures [Work](TASK) under pressure [Communicate](TASK) [present](TASK) and [report](TASK) to relevant stakeholders [Manage](TASK) and [analyse](TASK) [log files](SKILLS)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>['Collect', 'Communicate', 'Manage', 'Practice', 'Work', 'analyse', 'correlate', 'present', 'report']</t>
+          <t>Incident handling [standards methodologies](SKILLS) and [frameworks](SKILLS) Incident handling [recommendations](SKILLS) and [best practices](SKILLS) Incident handling tools Incident handling [communication procedures](SKILLS) [Operating systems](SKILLS) [security](SKILLS) Computer [networks security](SKILLS) [Cyber threats](SKILLS) [Cybersecurity attack pr[ocedur](TASK)es](SKILLS) Computer [systems](SKILLS) [vulnerabilities](SKILLS) [Cybersecurity](SKILLS)-related [certifications](SKILLS) [Cybersecurity](SKILLS) related [laws regulations](SKILLS) and legislations [Secure][(TASK) Operation Centres](SKILLS) (SOCs) operation Computer [Security](SKILLS) Incident [Response](TASK) Teams (CSIRTs) operation</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>['Cybersecurity', 'Management practices', 'Resource management', 'Risk management', 'best practices', 'certifications', 'clouds', 'cybersecurity', 'frameworks', 'infrastructures', 'log files', 'methodologies', 'operating systems', 'operational aspects', 'recommendations', 'servers', 'stakeholders', 'systems']</t>
+          <t>['Analyses', 'Communicate', 'Manage', 'Practice', 'Response', 'Secure', 'Work', 'analyse', 'attack', 'correlate', 'evaluates', 'present', 'processes', 'report', 'response']</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>['Cyber threats', 'Cybersecurity', 'Cybersecurity attack procedures', 'Cybersecurity standards methodologies', 'Management practices', 'Operating systems', 'Resource management', 'Risk management', 'Secure Operation Centres', 'Security', 'best practices', 'certifications', 'clouds', 'communication procedures', 'cyber', 'cyber threat', 'cybersecurity', 'cybersecurity incidents', 'frameworks', 'laws regulations', 'log files', 'networks security', 'operating systems', 'operational', 'operational aspects', 'policies', 'recommendations', 'security', 'standards methodologies', 'systems', 'vulnerabilities']</t>
         </is>
       </c>
     </row>
@@ -692,7 +638,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Oversees and assures compliance with cybersecurity- and data-related legal, regulatory frameworks and policies in line with the organisation’s strategy and legal requirements. Contributes to the organisation’s data protection related actions. Provides legal advice in the development of the organisation’s cybersecurity governance processes and recommended remediation strategies/solutions to ensure compliance.</t>
+          <t>Oversees and assures compliance with cybersecurity- and data-related legal regulatory frameworks and policies in line with the organisation’s strategy and legal requirements. Contributes to the organisation’s data protection related actions. Provides legal advice in the development of the organisation’s cybersecurity governance processes and recommended remediation strategies/solutions to ensure compliance.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -703,85 +649,47 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Ensure compliance with and provide legal advice and guidance on data privacy and  data protection standards, laws and regulations 
- Identify and document compliance gaps 
- Conduct privacy impact assessments and develop, maintain, communicate and train  upon the privacy policies, procedures 
- Enforce and advocate organisation’s data privacy and protection program 
- Ensure that data owners, holders, controllers, processors, subjects, internal or  external partners and entities are informed about their data protection rights,  obligations and responsibilities 
- Act as a key contact point to handle queries and complaints regarding data  processing 
- Assist in designing, implementing, auditing and compliance testing activities in order  to ensure cybersecurity and privacy compliance 
- Monitor audits and data protection related training activities 
- Cooperate and share information with authorities and professional groups 
- Contribute to the development of the organisation’s cybersecurity strategy, policy  and procedures 
- Develop and propose staff awareness training to achieve compliance and foster a  culture of data protection within the organization 
- Manage legal aspects of information security responsibilities and third-party relations</t>
+          <t>Ensure compliance with and provide legal advice and guidance on data privacy and data protection standards laws and regulations Identify and document compliance gaps Conduct privacy impact assessments and develop maintain communicate and train upon the privacy policies procedures Enforce and advocate organisation’s data privacy and protection program Ensure that data owners holders controllers processors subjects internal or external partners and entities are informed about their data protection rights obligations and responsibilities Act as a key contact point to handle queries and complaints regarding data processing Assist in designing implementing auditing and compliance testing activities in order to ensure cybersecurity and privacy compliance Monitor audits and data protection related training activities Cooperate and share information with authorities and professional groups Contribute to the development of the organisation’s cybersecurity strategy policy and procedures Develop and propose staff awareness training to achieve compliance and foster a culture of data protection within the organization Manage legal aspects of information security responsibilities and third-party relations</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Comprehensive understanding of the business strategy, models and products and  ability to factor into legal, regulatory and standards’ requirements 
- Carry out working-life practices of the data protection and privacy issues involved in  the implementation of the organisational processes, finance and business strategy 
- Lead the development of appropriate cybersecurity and privacy policies and  procedures that complement the business needs and legal requirements; further  ensure its acceptance, comprehension and implementation and communicate it  between the involved parties 
- Conduct, monitor and review privacy impact assessments using standards,  frameworks, acknowledged methodologies and tools 
- Explain and communicate data protection and privacy topics to stakeholders and  users 
- Understand, practice and adhere to ethical requirements and standards 
- Understand legal framework modifications implications to the organisation’s  cybersecurity and data protection strategy and policies 
- Collaborate with other team members and colleague
-</t>
+          <t>Comprehensive understanding of the business strategy models and products and ability to factor into legal regulatory and standards’ requirements Carry out working-life practices of the data protection and privacy issues involved in the implementation of the organisational processes finance and business strategy Lead the development of appropriate cybersecurity and privacy policies and procedures that complement the business needs and legal requirements; further ensure its acceptance comprehension and implementation and communicate it between the involved parties Conduct monitor and review privacy impact assessments using standards frameworks acknowledged methodologies and tools Explain and communicate data protection and privacy topics to stakeholders and users Understand practice and adhere to ethical requirements and standards Understand legal framework modifications implications to the organisation’s cybersecurity and data protection strategy and policies Collaborate with other team members and colleague</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Cybersecurity related laws, regulations and legislations
- Cybersecurity standards, methodologies and frameworks 
- Cybersecurity policies 
- Legal, regulatory and legislative compliance requirements, recommendations and  best practices 
- Privacy impact assessment standards, methodologies and frameworks
-</t>
+          <t>Cybersecurity related laws regulations and legislations Cybersecurity standards methodologies and frameworks Cybersecurity policies Legal regulatory and legislative compliance requirements recommendations and best practices Privacy impact assessment standards methodologies and frameworks</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Oversees and assures compliance with [cybersecurity](SKILLS)- and data-related legal, [regulatory frameworks](SKILLS) and policies in line with the organisation’s strategy and legal requirements. Contributes to the organisation’s [data protection](SKILLS) related actions. Provides [legal advice](SKILLS) in the development of the organisation’s [cybersecurity](SKILLS) [governance processes](SKILLS) and recommended [remediation strategies](SKILLS)/[solutions](SKILLS) to [ensure](TASK) compliance.</t>
+          <t>Oversees and assures compliance with [cybersecurity](SKILLS)- and [data](SKILLS)-related [legal regulatory frameworks](SKILLS) and [policies](SKILLS) in line with the organisation’s [strategy](SKILLS) and [legal](SKILLS) requirements. Contributes to the organisation’s [data protection](SKILLS) related actions. Provides [legal advice](SKILLS) in the development of the organisation’s [cybersecurity](SKILLS) [governance processes[](SKILLS)](TASK) and recommended [remediation strategies](SKILLS)/[solutions](SKILLS) to [ensure](TASK) compliance.</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t xml:space="preserve"> [Ensure](TASK) compliance with and [provide](TASK) [legal advice](SKILLS) and guidance on [data privacy](SKILLS) and  [data protection](SKILLS) standards, laws and regulations 
- [Identify](TASK) and [document](TASK) [compliance gaps](SKILLS) 
- [Conduct](TASK) privacy impact assessments and [develop](TASK), [maintain](TASK), [communicate](TASK) and [train](TASK)  upon the [privacy policies](SKILLS), procedures 
- [Enforce](TASK) and [advocate](TASK) organisation’s [data privacy](SKILLS) and protection program 
- [Ensure](TASK) that data owners, holders, controllers, processors, subjects, internal or  external partners and entities are informed about their [data protection](SKILLS) rights,  obligations and responsibilities 
- Act as a key contact point to [handle](TASK) queries and complaints regarding data  processing 
- [Assist](TASK) in designing, implementing, auditing and [compliance testing](SKILLS) activities in order  to [ensure](TASK) [cybersecurity](SKILLS) and privacy compliance 
- [Monitor](TASK) audits and [data protection](SKILLS) related [training activities](SKILLS) 
- Cooperate and [share](TASK) information with authorities and professional groups 
- [Contribute](TASK) to the development of the organisation’s [cybersecurity](SKILLS) strategy, policy  and procedures 
- [Develop](TASK) and [propose](TASK) [staff awareness](SKILLS) training to achieve compliance and foster a  culture of [data protection](SKILLS) within the organization 
- [Manage](TASK) legal aspects of information security responsibilities and third-party relations</t>
+          <t>[Ensure](TASK) compliance with and [provide](TASK) [legal advice](SKILLS) and guidance on [data privacy](SKILLS) and [data protection](SKILLS) standards [laws](SKILLS) and regulations [Identify](TASK) and [document](TASK) [compliance gaps](SKILLS) [Conduct](TASK) privacy impact assessments and [develop](TASK) [maintain](TASK) [communicate](TASK) and [train](TASK) upon the [privacy policies](SKILLS) procedures [Enforce](TASK) and advocate organisation’s [data privacy](SKILLS) and [protection program](SKILLS) [Ensure](TASK) that [data](SKILLS) owners holders controllers processors subjects internal or external partners and entities are informed about their [data protection](SKILLS) rights obligations and responsibilities Act as a key contact point to [handle](TASK) queries and complaints regarding [data processing](SKILLS) [Assist](TASK) in designing implementing auditing and [compliance testing]([SKILLS)](TASK) activities in order to [ensure](TASK) [cybersecurity](SKILLS) and [privacy compliance](SKILLS) [Monitor](TASK) audits and [data protection](SKILLS) related [training activities](SKILLS) [Cooperate](TASK) and [share](TASK) information with authorities and professional groups [Contribute](TASK) to the development of the organisation’s [cybersecurity strategy](SKILLS) [policy](SKILLS) and procedures [Develop](TASK) and [propose](TASK) staff [awareness training](SKILLS) to achieve compliance and foster a culture of [data protection](SKILLS) within the organization [Manage](TASK) [legal aspects](SKILLS) of [information security](SKILLS) responsibilities and third-party relations</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Comprehensive understanding of the [business strategy](SKILLS), models and [products](SKILLS) and  ability to factor into legal, regulatory and standards’ requirements 
- Carry out [working-life practices](SKILLS) of the [data protection](SKILLS) and privacy issues involved in  the [implementation](SKILLS) of the organisational processes, finance and [business strategy](SKILLS) 
- [Lead](TASK) the development of appropriate [cybersecurity](SKILLS) and [privacy policies](SKILLS) and  procedures that complement the business needs and legal requirements; further  [ensure](TASK) its acceptance, comprehension and [implementation](SKILLS) and [communicate](TASK) it  between the involved parties 
- [Conduct](TASK), [monitor](TASK) and [review](TASK) privacy impact assessments using standards,  [frameworks](SKILLS), acknowledged [methodologies](SKILLS) and tools 
- [Explain](TASK) and [communicate](TASK) [data protection](SKILLS) and privacy topics to [stakeholders](SKILLS) and  users 
- Understand, [practice](TASK) and adhere to [ethical requirements](SKILLS) and standards 
- Understand [legal framework](SKILLS) modifications implications to the organisation’s  [cybersecurity](SKILLS) and [data protection](SKILLS) strategy and policies 
- [Collaborate](TASK) with other team members and colleague
-</t>
+          <t>Comprehensive understanding of the [business strategy](SKILLS) models and [products](SKILLS) and [ability](TASK) to factor into [legal regulatory](SKILLS) and standards’ requirements Carry out [working-life practices](SKILLS) of the [data protection](SKILLS) and privacy issues involved in the [implementation](SKILLS) of the organisational [processes](TASK) finance and [business strategy](SKILLS) [Lead](TASK) the development of appropriate [cybersecurity](SKILLS) and [privacy policies](SKILLS) and procedures that complement the business needs and [legal](SKILLS) requirements; further [ensure](TASK) its acceptance comprehension and [implementation](SKILLS) and [communicate](TASK) it between the involved parties [Conduct](TASK) [monitor](TASK) and [review](TASK) privacy impact assessments using standards [frameworks](SKILLS) acknowledged [methodologies](SKILLS) and tools [Explain](TASK) and [communicate](TASK) [data protection](SKILLS) and privacy topics to stakeholders and users Understand [practice](TASK) and adhere to [ethical requirements](SKILLS) and standards Understand [legal framework](SKILLS) modifications implications to the organisation’s [cybersecurity](SKILLS) and [data protection](SKILLS) [strategy](SKILLS) and [policies](SKILLS) [Collaborate](TASK) with other team members and colleague</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>['Assist', 'Collaborate', 'Conduct', 'Contribute', 'Develop', 'Enforce', 'Ensure', 'Explain', 'Identify', 'Lead', 'Manage', 'Monitor', 'advocate', 'communicate', 'develop', 'document', 'ensure', 'handle', 'maintain', 'monitor', 'practice', 'propose', 'provide', 'review', 'share', 'train']</t>
+          <t>[Cybersecurity](SKILLS) related [laws regulations](SKILLS) and legislations [Cybersecurity standards methodologies](SKILLS) and [frameworks](SKILLS) [Cybersecurity](SKILLS) [policies](SKILLS) [Legal regulatory](SKILLS) and legislative compliance requirements [recommendations](SKILLS) and [best practices](SKILLS) Privacy impact assessment [standards methodologies](SKILLS) and [frameworks](SKILLS)</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>['business strategy', 'compliance gaps', 'compliance testing', 'cybersecurity', 'data privacy', 'data protection', 'ethical requirements', 'frameworks', 'governance processes', 'implementation', 'legal advice', 'legal framework', 'methodologies', 'privacy policies', 'products', 'regulatory frameworks', 'remediation strategies', 'solutions', 'staff awareness', 'stakeholders', 'training activities', 'working-life practices']</t>
+          <t>['Assist', 'Collaborate', 'Conduct', 'Contribute', 'Cooperate', 'Develop', 'Enforce', 'Ensure', 'Explain', 'Identify', 'Lead', 'Manage', 'Monitor', 'ability', 'communicate', 'develop', 'document', 'ensure', 'handle', 'maintain', 'monitor', 'practice', 'processes', 'propose', 'provide', 'review', 'share', 'testing', 'train']</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>['Cybersecurity', 'Cybersecurity standards methodologies', 'Legal regulatory', 'awareness training', 'best practices', 'business strategy', 'compliance gaps', 'compliance testing', 'cybersecurity', 'cybersecurity strategy', 'data', 'data privacy', 'data processing', 'data protection', 'ethical requirements', 'frameworks', 'governance processes', 'implementation', 'information security', 'laws', 'laws regulations', 'legal', 'legal advice', 'legal aspects', 'legal framework', 'legal regulatory', 'legal regulatory frameworks', 'methodologies', 'policies', 'policy', 'privacy compliance', 'privacy policies', 'products', 'protection program', 'recommendations', 'remediation strategies', 'solutions', 'standards methodologies', 'strategy', 'training activities', 'working-life practices']</t>
         </is>
       </c>
     </row>
@@ -796,7 +704,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Manages cyber threat intelligence life cycle including cyber threat information  collection, analysis and production of actionable intelligence and dissemination to  security stakeholders and the CTI community, at a tactical, operational and strategic  level. Identifies and monitors the Tactics, Techniques and Procedures (TTPs) used  by cyber threat actors and their trends, track threat actors’ activities and observe how  non-cyber events can influence cyber-related actions.</t>
+          <t>Manages cyber threat intelligence life cycle including cyber threat information collection analysis and production of actionable intelligence and dissemination to security stakeholders and the CTI community at a tactical operational and strategic level. Identifies and monitors the Tactics Techniques and Procedures (TTPs) used by cyber threat actors and their trends track threat actors’ activities and observe how non-cyber events can influence cyber-related actions.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -807,99 +715,47 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Develop, implement and manage the organisation's cyber threat intelligence  strategy 
- Develop plans and procedures to manage threat intelligence 
- Translate business requirements into Intelligence Requirements 
- Implement threat intelligence collection, analysis and production of actionable  intelligence and dissemination to security stakeholders 
- Identify and assess cyber threat actors targeting the organisation 
- Identify, monitor and assess the Tactics, Techniques and Procedures (TTPs) used  by cyber threat actors by analysing open-source and proprietary data, information  and intelligence 
- Produce actionable reports based on threat intelligence data 
- Elaborate and advise on mitigation plans at the tactical, operational and strategic  level 
- Coordinate with stakeholders to share and consume intelligence on relevant cyber  threats 
- Leverage intelligence data to support and assist with threat modelling,  recommendations for Risk Mitigation and cyber threat hunting 
- Articulate and communicate intelligence openly and publicly at all levels 
- Convey the proper security severity by explaining the risk exposure and its  consequences to non-technical stakeholders
-</t>
+          <t>Develop implement and manage the organisation's cyber threat intelligence strategy Develop plans and procedures to manage threat intelligence Translate business requirements into Intelligence Requirements Implement threat intelligence collection analysis and production of actionable intelligence and dissemination to security stakeholders Identify and assess cyber threat actors targeting the organisation Identify monitor and assess the Tactics Techniques and Procedures (TTPs) used by cyber threat actors by analysing open-source and proprietary data information and intelligence Produce actionable reports based on threat intelligence data Elaborate and advise on mitigation plans at the tactical operational and strategic level Coordinate with stakeholders to share and consume intelligence on relevant cyber threats Leverage intelligence data to support and assist with threat modelling recommendations for Risk Mitigation and cyber threat hunting Articulate and communicate intelligence openly and publicly at all levels Convey the proper security severity by explaining the risk exposure and its consequences to non-technical stakeholders</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Collaborate with other team members and colleagues 
- Collect, analyse and correlate cyber threat information originating from multiple  sources 
- Identify threat actors TTPs and campaigns 
- Automate threat intelligence management procedures 
- Conduct technical analysis and reporting 
- Identify non-cyber events with implications on cyber-related activities 
- Model threats, actors and TTPs 
- Communicate, coordinate and cooperate with internal and external stakeholders 
- Communicate, present and report to relevant stakeholders 
- Use and apply CTI platforms and tools
-</t>
+          <t>Collaborate with other team members and colleagues Collect analyse and correlate cyber threat information originating from multiple sources Identify threat actors TTPs and campaigns Automate threat intelligence management procedures Conduct technical analysis and reporting Identify non-cyber events with implications on cyber-related activities Model threats actors and TTPs Communicate coordinate and cooperate with internal and external stakeholders Communicate present and report to relevant stakeholders Use and apply CTI platforms and tools</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Operating systems security 
- Computer networks security 
- Cybersecurity controls and solutions 
- Computer programming 
- Cyber Threat Intelligence (CTI) sharing standards, methodologies and frameworks 
- Responsible information disclosure procedures 
- Cross-domain and border-domain knowledge related to cybersecurity 
- Cyber threats 
- Cyber threat actors 
- Cybersecurity attack procedures 
- Advanced and persistent cyber threats (APT) 
- Threat actors Tactics, Techniques and Procedures (TTPs) 
- Cybersecurity-related certifications
-</t>
+          <t>Operating systems security Computer networks security Cybersecurity controls and solutions Computer programming Cyber Threat Intelligence (CTI) sharing standards methodologies and frameworks Responsible information disclosure procedures Cross-domain and border-domain knowledge related to cybersecurity Cyber threats Cyber threat actors Cybersecurity attack procedures Advanced and persistent cyber threats (APT) Threat actors Tactics Techniques and Procedures (TTPs) Cybersecurity-related certifications</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Manages cyber threat intelligence life cycle including cyber threat information  collection, analysis and production of actionable intelligence and dissemination to  security [stakeholders](SKILLS) and the CTI community, at a tactical, operational and strategic  level. Identifies and monitors the Tactics, Techniques and Procedures (TTPs) used  by cyber [threat actors](SKILLS) and their trends, [track](TASK) [threat actors](SKILLS)’ activities and observe how  [non-cyber events](SKILLS) can influence cyber-related actions.</t>
+          <t>[Manages](TASK) [cyber threat intelligence](SKILLS) life cycle including [cyber threat](SKILLS) information collection analysis and production of actionable intelligence and dissemination to [security](SKILLS) stakeholders and the CTI community at a tactical [operational](SKILLS) and strategic level. Identifies and monitors the [Tactics Technique[s and Proc](TASK)edures](SKILLS) (TTPs) used by [cyber threat](SKILLS) actors and their trends [track](TASK) threat actors’ activities and observe how [non-cyber events](SKILLS) can influence [cyber](SKILLS)-related actions.</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> [Develop](TASK), [implement](TASK) and [manage](TASK) the organisation's cyber threat intelligence  strategy 
- [Develop](TASK) plans and procedures to [manage](TASK) threat intelligence 
- [Translate](TASK) business requirements into [Intelligence Requirements](SKILLS) 
- [Implement](TASK) threat intelligence collection, analysis and production of actionable  intelligence and dissemination to security [stakeholders](SKILLS) 
- [Identify](TASK) and [assess](TASK) cyber [threat actors](SKILLS) targeting the organisation 
- [Identify](TASK), [monitor](TASK) and [assess](TASK) the Tactics, Techniques and Procedures (TTPs) used  by cyber [threat actors](SKILLS) by analysing open-source and proprietary data, information  and intelligence 
- [Produce](TASK) actionable reports based on threat intelligence data 
- [Elaborate](TASK) and [advise](TASK) on mitigation plans at the tactical, operational and strategic  level 
- [Coordinate](TASK) with [stakeholders](SKILLS) to [share](TASK) and consume intelligence on relevant cyber  threats 
- [Leverage](TASK) intelligence data to [support[](TASK)](SKILLS) and [assist](TASK) with threat modelling,  [recommendations](SKILLS) for [Risk Mitigation](SKILLS) and [cyber threat hunting](SKILLS) 
- [Articulate](TASK) and [communicate](TASK) intelligence openly and publicly at all levels 
- [Convey](TASK) the proper security severity by explaining the risk exposure and its  consequences to non-technical [stakeholders](SKILLS)
-</t>
+          <t>[Develop](TASK) [implement](TASK) and [manage](TASK) the organisation's [cyber threat intelligence strategy](SKILLS) [Develop](TASK) plans and procedures to [manage](TASK) threat intelligence [Translate](TASK) business requirements into [Intelligence Requirements](SKILLS) [Implement](TASK) threat intelligence collection analysis and production of actionable intelligence and dissemination to [security](SKILLS) stakeholders [Identify](TASK) and [assess](TASK) [cyber threat](SKILLS) actors targeting the organisation [Identify](TASK) [monitor](TASK) and [assess](TASK) the [Tactics Technique[s and Proc](TASK)edures](SKILLS) (TTPs) used by [cyber threat](SKILLS) actors by analysing [open-source](SKILLS) and proprietary [data](SKILLS) information and intelligence [Produce](TASK) [actionable reports](SKILLS) based on threat intelligence [data](SKILLS) [Elaborate](TASK) and [advise](TASK) on mitigation plans at the tactical [operational](SKILLS) and strategic level [Coordinate](TASK) with stakeholders to [share](TASK) and consume intelligence on relevant [cyber threats](SKILLS) [Leverage](TASK) intelligence [data](SKILLS) to [support](TASK) and [assist](TASK) with threat modelling [recommendations](SKILLS) for Risk Mitigation and [cyber threat hunting](SKILLS) [Articulate](TASK) and [communicate](TASK) intelligence openly and publicly at all levels [Convey](TASK) the proper [security](SKILLS) severity by explaining the risk exposure and its consequences to non-technical stakeholders</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> [Collaborate](TASK) with other team members and [colleagues](SKILLS) 
- [Collect](TASK), [analyse](TASK) and [correlate](TASK) cyber threat information originating from multiple  sources 
- [Identify](TASK) [threat actors](SKILLS) TTPs and campaigns 
- [Automate](TASK) threat intelligence management procedures 
- [Conduct](TASK) [technical analysis](SKILLS) and reporting 
- [Identify](TASK) [non-cyber events](SKILLS) with implications on cyber-related activities 
- [Model](TASK) threats, actors and TTPs 
- [Communicate](TASK), [coordinate](TASK) and cooperate with internal and external [stakeholders](SKILLS) 
- [Communicate](TASK), [present](TASK) and [report](TASK) to relevant [stakeholders](SKILLS) 
- [Use](TASK) and [apply](TASK) [CTI platforms](SKILLS) and tools
-</t>
+          <t>[Collaborate](TASK) with other team members and colleagues Collect [analyse](TASK) and [correlate](TASK) [cyber threat](SKILLS) information originating from multiple sources [Identify](TASK) threat actors TTPs and campaigns [Automate](TASK) [threat intelligence management](SKILLS) procedures [Conduct](TASK) [technical analysis](SKILLS) and reporting [Identify](TASK) [non-cyber events](SKILLS) with implications on [cyber-related activities](SKILLS) [Model](TASK) threats actors and TTPs [Communicate](TASK) [coordinate](TASK) and [cooperate](TASK) with internal and external stakeholders [Communicate](TASK) [present](TASK) and [report](TASK) to relevant stakeholders [Use](TASK) and [apply](TASK) [CTI platforms](SKILLS) and tools</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>['Articulate', 'Automate', 'Collaborate', 'Collect', 'Communicate', 'Conduct', 'Convey', 'Coordinate', 'Develop', 'Elaborate', 'Identify', 'Implement', 'Leverage', 'Model', 'Produce', 'Translate', 'Use', 'advise', 'analyse', 'apply', 'assess', 'assist', 'communicate', 'coordinate', 'correlate', 'implement', 'manage', 'monitor', 'present', 'report', 'share', 'support', 'track']</t>
+          <t>[Operating systems](SKILLS) [security](SKILLS) Computer [networks security](SKILLS) [Cybersecurity](SKILLS) [controls](SKILLS) and [solutions](SKILLS) Computer [programming](TASK) [Cyber Threat Intelligence](SKILLS) (CTI) sharing [standards methodologies](SKILLS) and [frameworks](SKILLS) Responsible information disclosure procedures Cross-domain and border-domain knowledge related to [cybersecurity](SKILLS) [Cyber threats](SKILLS) [Cyber threat](SKILLS) actors [Cybersecurity attack pr[ocedur](TASK)es](SKILLS) Advanced and persistent [cyber threats](SKILLS) (APT) Threat actors [Tactics Technique[s and Proc](TASK)edures](SKILLS) (TTPs) [Cybersecurity](SKILLS)-related [certifications](SKILLS)</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>['CTI platforms', 'Intelligence Requirements', 'Risk Mitigation', 'colleagues', 'cyber threat hunting', 'non-cyber events', 'recommendations', 'stakeholders', 'support', 'technical analysis', 'threat actors']</t>
+          <t>['Articulate', 'Automate', 'Collaborate', 'Communicate', 'Conduct', 'Convey', 'Coordinate', 'Develop', 'Elaborate', 'Identify', 'Implement', 'Leverage', 'Manages', 'Model', 'Produce', 'Techniques', 'Translate', 'Use', 'advise', 'analyse', 'apply', 'assess', 'assist', 'attack', 'communicate', 'cooperate', 'coordinate', 'correlate', 'implement', 'manage', 'monitor', 'present', 'programming', 'report', 'share', 'support', 'track']</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>['CTI platforms', 'Cyber Threat Intelligence', 'Cyber threat', 'Cyber threats', 'Cybersecurity', 'Cybersecurity attack procedures', 'Intelligence Requirements', 'Operating systems', 'Tactics Techniques and Procedures', 'actionable reports', 'certifications', 'controls', 'cyber', 'cyber threat', 'cyber threat hunting', 'cyber threat intelligence', 'cyber threat intelligence strategy', 'cyber threats', 'cyber-related activities', 'cybersecurity', 'data', 'frameworks', 'networks security', 'non-cyber events', 'open-source', 'operational', 'recommendations', 'security', 'solutions', 'standards methodologies', 'technical analysis', 'threat intelligence management']</t>
         </is>
       </c>
     </row>
@@ -914,7 +770,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Designs solutions based on security-by-design and privacy-by-design principles.  Creates and continuously improves architectural models and develops appropriate  architectural documentation and specifications. Coordinate secure development,  integration and maintenance of cybersecurity components in line with standards and  other related requirements</t>
+          <t>Designs solutions based on security-by-design and privacy-by-design principles. Creates and continuously improves architectural models and develops appropriate architectural documentation and specifications. Coordinate secure development integration and maintenance of cybersecurity components in line with standards and other related requirements</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -926,98 +782,47 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Design and propose a secure architecture to implement the organisation’s strategy  Develop organisation’s cybersecurity architecture to address security and privacy  requirements 
- Produce architectural documentation and specifications 
- Present high-level security architecture design to stakeholders 
- Establish a secure environment during the development lifecycle of systems,  services and products 
- Coordinate the development, integration and maintenance of cybersecurity  components ensuring the cybersecurity specifications 
- Analyse and evaluate the cybersecurity of the organisation’s architecture 
- Assure the security of the solution architectures through security reviews and  certification 
- Collaborate with other teams and colleagues 
- Evaluate the impact of cybersecurity solutions on the design  
-and performance of the organisation’s architecture 
- Adapt the organisation’s architecture to emerging threats 
- Assess the implemented architecture to maintain an appropriate level of security</t>
+          <t>Design and propose a secure architecture to implement the organisation’s strategy Develop organisation’s cybersecurity architecture to address security and privacy requirements Produce architectural documentation and specifications Present high-level security architecture design to stakeholders Establish a secure environment during the development lifecycle of systems services and products Coordinate the development integration and maintenance of cybersecurity components ensuring the cybersecurity specifications Analyse and evaluate the cybersecurity of the organisation’s architecture Assure the security of the solution architectures through security reviews and certification Collaborate with other teams and colleagues Evaluate the impact of cybersecurity solutions on the design and performance of the organisation’s architecture Adapt the organisation’s architecture to emerging threats Assess the implemented architecture to maintain an appropriate level of security</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Conduct user and business security requirements analysis 
- Draw cybersecurity architectural and functional specifications 
- Decompose and analyse systems to develop security and privacy requirements and  identify effective solutions 
- Design systems and architectures based on security and privacy by design and by  defaults cybersecurity principles 
- Guide and communicate with implementers and IT/OT personnel 
- Communicate, present and report to relevant stakeholders 
- Propose cybersecurity architectures based on stakeholder’s needs and budget 
- Select appropriate specifications, procedures and controls 
- Build resilience against points of failure across the architecture 
- Coordinate the integration of security solutions
-</t>
+          <t>Conduct user and business security requirements analysis Draw cybersecurity architectural and functional specifications Decompose and analyse systems to develop security and privacy requirements and identify effective solutions Design systems and architectures based on security and privacy by design and by defaults cybersecurity principles Guide and communicate with implementers and IT/OT personnel Communicate present and report to relevant stakeholders Propose cybersecurity architectures based on stakeholder’s needs and budget Select appropriate specifications procedures and controls Build resilience against points of failure across the architecture Coordinate the integration of security solutions</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Cybersecurity-related certifications 
- Cybersecurity recommendations and best practices 
- Cybersecurity standards, methodologies and frameworks 
- Cybersecurity-related requirements analysis 
- Secure development lifecycle 
- Security architecture reference models 
- Cybersecurity-related technologies 
- Cybersecurity controls and solutions 
- Cybersecurity risks 
- Cyber threats 
- Cybersecurity trends 
- Legal, regulatory and legislative compliance requirements, recommendations and  best practices 
- Legacy cybersecurity procedures 
- Privacy-Enhancing Technologies (PET)
-</t>
+          <t>Cybersecurity-related certifications Cybersecurity recommendations and best practices Cybersecurity standards methodologies and frameworks Cybersecurity-related requirements analysis Secure development lifecycle Security architecture reference models Cybersecurity-related technologies Cybersecurity controls and solutions Cybersecurity risks Cyber threats Cybersecurity trends Legal regulatory and legislative compliance requirements recommendations and best practices Legacy cybersecurity procedures Privacy-Enhancing Technologies (PET)</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Designs [solutions](SKILLS) based on [security-by-design](S[KILLS)](TASK) and [privacy-by-design](S[KILLS)](TASK) principles.  Creates and continuously improves [architectural models](SKILLS) and develops appropriate  [architectural documentation](SKILLS) and specifications. [Coordinate](TASK) [secure](TASK) development,  [integration](SKILLS) and maintenance of [cybersecurity](SKILLS) components in line with standards and  other related requirements</t>
+          <t>Designs [solutions](SKILLS) based on [security-by-design](S[KILLS)](TASK) and [privacy-by-design](S[KILLS)](TASK) principles. Creates and continuously improves [architectural models](SKILLS) and develops appropriate [architectural documentation](SKILLS) and specifications. [Coordinate](TASK) [secure][(TASK) development](SKILLS) [integration](SKILLS) and maintenance of [cybersecurity](SKILLS) components in line with standards and other related requirements</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t xml:space="preserve"> [Design](TASK) and [propose](TASK) a [secure](TASK) architecture to [implement](TASK) the organisation’s strategy  [Develop](TASK) organisation’s [cybersecurity](SKILLS) architecture to address security and privacy  requirements 
- [Produce](TASK) [architectural documentation](SKILLS) and specifications 
- [Present](TASK) [high-level security architecture](SKILLS) [design](TASK) to [stakeholders](SKILLS) 
- [Establish](TASK) a [secure](TASK) environment during the development lifecycle of [systems](SKILLS),  [services](SKILLS) and [products](SKILLS) 
- [Coordinate](TASK) the development, [integration](SKILLS) and maintenance of [cybersecurity](SKILLS)  components ensuring the [cybersecurity](SKILLS) specifications 
- [Analyse](TASK) and [evaluate](TASK) the [cybersecurity](SKILLS) of the organisation’s architecture 
- [Assure](TASK) the security of the [solution architectures](SKILLS) through [security reviews](SKILLS) and  certification 
- [Collaborate](TASK) with other teams and [colleagues](SKILLS) 
- [Evaluate](TASK) the impact of [cybersecurity](SKILLS) [solutions](SKILLS) on the [design](TASK)  
-and performance of the organisation’s architecture 
- [Adapt](TASK) the organisation’s architecture to [emerging threats](SKILLS) 
- [Assess](TASK) the implemented architecture to [maintain](TASK) an appropriate level of security</t>
+          <t>[Design](TASK) and [propose](TASK) a [secure][(TASK) architecture](SKILLS) to [implement](TASK) the organisation’s [strategy](SKILLS) [Develop](TASK) organisation’s [cybersecurity](SKILLS) [architecture](SKILLS) to address [security](SKILLS) and privacy requirements [Produce](TASK) [architectural documentation](SKILLS) and specifications [Present](TASK) [high-level security architecture](SKILLS) [design](TASK) to stakeholders [Establish](TASK) a [secure](TASK) environment during the development lifecycle of [systems](SKILLS) [services](SKILLS) and [products](SKILLS) [Coordinate](TASK) the development [integration](SKILLS) and maintenance of [cybersecurity](SKILLS) components ensuring the [cybersecurity](SKILLS) specifications [Analyse](TASK) and [evaluate](TASK) the [cybersecurity](SKILLS) of the organisation’s [architecture](SKILLS) [Assure](TASK) the [security](SKILLS) of the [solution architectures](SKILLS) through [security reviews](SKILLS) and certification [Collaborate](TASK) with other teams and colleagues [Evaluate](TASK) the impact of [cybersecurity](SKILLS) [solutions](SKILLS) on the [design](TASK) and performance of the organisation’s [architecture](SKILLS) [Adapt](TASK) the organisation’s [architecture](SKILLS) to [emerging threats](SKILLS) [Assess](TASK) the [implemented](TASK) [architecture](SKILLS) to [maintain](TASK) an appropriate level of [security](SKILLS)</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t xml:space="preserve"> [Conduct](TASK) user and business security requirements analysis 
- [Draw](TASK) [cybersecurity](SKILLS) architectural and [functional specifications](SKILLS) 
- [Decompose](TASK) and [analyse](TASK) [systems](SKILLS) to [develop](TASK) security and privacy requirements and  [identify](TASK) [effective solutions](SKILLS) 
- [Design](TASK) [systems](SKILLS) and architectures based on security and privacy by [design](TASK) and by  defaults [cybersecurity](SKILLS) principles 
- [Guide](TASK) and [communicate](TASK) with implementers and IT/OT personnel 
- [Communicate](TASK), [present](TASK) and [report](TASK) to relevant [stakeholders](SKILLS) 
- [Propose](TASK) [cybersecurity](SKILLS) architectures based on stakeholder’s needs and budget 
- [Select](TASK) appropriate specifications, procedures and [controls](SKILLS) 
- [Build](TASK) [resilience](SKILLS) against [points of failure](SKILLS) across the architecture 
- [Coordinate](TASK) the [integration of security solutions](SKILLS)
-</t>
+          <t>[Conduct](TASK) user and [business security requirements](SKILLS) analysis [Draw](TASK) [cybersecurity architectural](SKILLS) and [functional specifications](SKILLS) [Decompose](TASK) and [analyse](TASK) [systems](SKILLS) to [develop](TASK) [security](SKILLS) and privacy requirements and [identify](TASK) [effective solutions](SKILLS) [Design](TASK) [systems](SKILLS) and architectures based on [security](SKILLS) and privacy by [design](TASK) and by defaults [cybersecurity](SKILLS) principles [Guide](TASK) and [communicate](TASK) with implementers and IT/OT personnel [Communicate](TASK) [present](TASK) and [report](TASK) to relevant stakeholders [Propose](TASK) [cybersecurity](SKILLS) architectures based on stakeholder’s needs and budget [Select](TASK) appropriate specifications procedures and [controls](SKILLS) [Build](TASK) [resilience](SKILLS) against [points of failure](SKILLS) across the [architecture](SKILLS) [Coordinate](TASK) the [integration of security solutions](SKILLS)</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>['Adapt', 'Analyse', 'Assess', 'Assure', 'Build', 'Collaborate', 'Communicate', 'Conduct', 'Coordinate', 'Decompose', 'Design', 'Develop', 'Draw', 'Establish', 'Evaluate', 'Guide', 'Present', 'Produce', 'Propose', 'Select', 'analyse', 'communicate', 'design', 'develop', 'evaluate', 'identify', 'implement', 'maintain', 'present', 'propose', 'report', 'secure']</t>
+          <t>[Cybersecurity](SKILLS)-related [certifications](SKILLS) [Cybersecurity](SKILLS) [recommendations](SKILLS) and [best practices](SKILLS) [Cybersecurity standards methodologies](SKILLS) and [frameworks](SKILLS) [Cybersecurity](SKILLS)-related requirements analysis [Secure][(TASK) development](SKILLS) lifecycle [Security architecture](SKILLS) reference models [Cybersecurity-related technologies](SKILLS) [Cybersecurity](SKILLS) [controls](SKILLS) and [solutions](SKILLS) [Cybersecurity risks](SKILLS) [Cyber threats](SKILLS) [Cybersecurity](SKILLS) trends [Legal regulatory](SKILLS) and legislative compliance requirements [recommendations](SKILLS) and [best practices](SKILLS) Legacy [cybersecurity](SKILLS) procedures Privacy-[Enhancing](TASK) Technologies (PET)</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>['architectural documentation', 'architectural models', 'colleagues', 'controls', 'cybersecurity', 'effective solutions', 'emerging threats', 'functional specifications', 'high-level security architecture', 'integration', 'integration of security solutions', 'points of failure', 'privacy-by-design', 'products', 'resilience', 'security reviews', 'security-by-design', 'services', 'solution architectures', 'solutions', 'stakeholders', 'systems']</t>
+          <t>['Adapt', 'Analyse', 'Assess', 'Assure', 'Build', 'Collaborate', 'Communicate', 'Conduct', 'Coordinate', 'Decompose', 'Design', 'Develop', 'Draw', 'Enhancing', 'Establish', 'Evaluate', 'Guide', 'Present', 'Produce', 'Propose', 'Secure', 'Select', 'analyse', 'communicate', 'design', 'develop', 'evaluate', 'identify', 'implement', 'implemented', 'maintain', 'present', 'propose', 'report', 'secure']</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>['Cyber threats', 'Cybersecurity', 'Cybersecurity risks', 'Cybersecurity standards methodologies', 'Cybersecurity-related technologies', 'Legal regulatory', 'Secure development', 'Security architecture', 'architectural documentation', 'architectural models', 'architecture', 'best practices', 'business security requirements', 'certifications', 'controls', 'cybersecurity', 'cybersecurity architectural', 'effective solutions', 'emerging threats', 'frameworks', 'functional specifications', 'high-level security architecture', 'integration', 'integration of security solutions', 'points of failure', 'privacy-by-design', 'products', 'recommendations', 'resilience', 'secure architecture', 'secure development', 'security', 'security reviews', 'security-by-design', 'services', 'solution architectures', 'solutions', 'strategy', 'systems']</t>
         </is>
       </c>
     </row>
@@ -1032,8 +837,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Conducts independent reviews to assess the effectiveness of processes and controls  and the overall compliance with the organisation's legal and regulatory frameworks  policies. Evaluates, tests and verifies cybersecurity-related products (systems,  hardware, software and services), functions and policies ensuring, compliance with  guidelines, standards and regulations.
-</t>
+          <t>Conducts independent reviews to assess the effectiveness of processes and controls and the overall compliance with the organisation's legal and regulatory frameworks policies. Evaluates tests and verifies cybersecurity-related products (systems hardware software and services) functions and policies ensuring compliance with guidelines standards and regulations.</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1044,91 +848,47 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Develop the organisation's auditing policy, procedures, standards and guidelines 
- Establish the methodologies and practices used for systems auditing 
- Establish the target environment and manage auditing activities 
- Define audit scope, objectives and criteria to audit against 
- Develop an audit plan describing the frameworks, standards, methodology,  procedures and auditing tests 
- Review target of evaluation, security objectives and requirements based on the risk  profile 
- Audit compliance with cybersecurity-related applicable laws and regulations 
- Audit conformity with cybersecurity-related applicable standards 
- Execute the audit plan and collect evidence and measurements 
- Maintain and protect the integrity of audit records 
- Develop and communicate conformity assessment, assurance, audit, certification  and maintenance reports 
- Monitor risk remediation activities
-</t>
+          <t>Develop the organisation's auditing policy procedures standards and guidelines Establish the methodologies and practices used for systems auditing Establish the target environment and manage auditing activities Define audit scope objectives and criteria to audit against Develop an audit plan describing the frameworks standards methodology procedures and auditing tests Review target of evaluation security objectives and requirements based on the risk profile Audit compliance with cybersecurity-related applicable laws and regulations Audit conformity with cybersecurity-related applicable standards Execute the audit plan and collect evidence and measurements Maintain and protect the integrity of audit records Develop and communicate conformity assessment assurance audit certification and maintenance reports Monitor risk remediation activities</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Organise and work in a systematic and deterministic way based on evidence 
- Follow and practice auditing frameworks, standards and methodologies 
- Apply auditing tools and techniques 
- Analyse business processes, assess and review software or hardware security, as  well as technical and organisational controls 
- Decompose and analyse systems to identify weaknesses and ineffective controls 
- Communicate, explain and adapt legal and regulatory requirements and business needs 
- Collect, evaluate, maintain and protect auditing information 
- Audit with integrity, being impartial and independent
-</t>
+          <t>Organise and work in a systematic and deterministic way based on evidence Follow and practice auditing frameworks standards and methodologies Apply auditing tools and techniques Analyse business processes assess and review software or hardware security as well as technical and organisational controls Decompose and analyse systems to identify weaknesses and ineffective controls Communicate explain and adapt legal and regulatory requirements and business needs Collect evaluate maintain and protect auditing information Audit with integrity being impartial and independent</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Cybersecurity controls and solutions 
- Legal, regulatory and legislative compliance requirements, recommendations and  best practices 
- Monitoring, testing and evaluating cybersecurity controls' effectiveness 
- Conformity assessment standards, methodologies and frameworks 
- Auditing standards, methodologies and frameworks 
- Cybersecurity standards, methodologies and frameworks 
- Auditing-related certification 
- Cybersecurity-related certifications
-</t>
+          <t>Cybersecurity controls and solutions Legal regulatory and legislative compliance requirements recommendations and best practices Monitoring testing and evaluating cybersecurity controls' effectiveness Conformity assessment standards methodologies and frameworks Auditing standards methodologies and frameworks Cybersecurity standards methodologies and frameworks Auditing-related certification Cybersecurity-related certifications</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Conducts independent reviews to [assess](TASK) the effectiveness of processes and [controls](SKILLS)  and the overall compliance with the organisation's legal and [regulatory frameworks](SKILLS)  policies. Evaluates, tests and verifies [cybersecurity](SKILLS)-related [products](SKILLS) ([systems](SKILLS),  hardware, software and [services](SKILLS)), functions and policies ensuring, compliance with  guidelines, standards and regulations.
-</t>
+          <t>Conducts independent reviews to [assess](TASK) the effectiveness of [processes](TASK) and [controls](SKILLS) and the overall compliance with the organisation's [legal](SKILLS) and [regulatory frameworks](SKILLS) [policies](SKILLS). [Evaluates](TASK) tests and verifies [cybersecurity](SKILLS)-related [products](SKILLS) ([systems](SKILLS) hardware software and [services](SKILLS)) functions and [policies](SKILLS) ensuring compliance with guidelines standards and regulations.</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t xml:space="preserve"> [Develop](TASK) the organisation's [auditing policy](SKILLS), procedures, standards and guidelines 
- [Establish](TASK) the [methodologies](SKILLS) and practices used for [systems auditing](SKILLS) 
- [Establish](TASK) the target environment and [manage](TASK) auditing activities 
- [Define](TASK) [audit]([TASK) scope](SKILLS), objectives and criteria to [audit](TASK) against 
- [Develop](TASK) an [audit](TASK) plan describing the [frameworks](SKILLS), standards, methodology,  procedures and auditing tests 
- [Review](TASK) target of evaluation, [security objectives](SKILLS) and requirements based on the risk  profile 
- [Audit](TASK) compliance with [cybersecurity](SKILLS)-related applicable laws and regulations 
- [Audit](TASK) conformity with [cybersecurity](SKILLS)-related applicable standards 
- Execute the [audit](TASK) plan and [collect](TASK) evidence and measurements 
- [Maintain](TASK) and [protect](TASK) the integrity of [audit](TASK) records 
- [Develop](TASK) and [communicate](TASK) [conformity assessment](SKILLS), assurance, [audit](TASK), certification  and [maintenance reports](SKILLS) 
- [Monitor](TASK) [risk remediation activities](SKILLS)
-</t>
+          <t>[Develop](TASK) the organisation's [auditing policy](SKILLS) procedures standards and guidelines [Establish](TASK) the [methodologies](SKILLS) and practices used for [systems auditing](SKILLS) [Establish](TASK) the target environment and [manage](TASK) auditing activities [Define](TASK) [audit]([TASK) scope](SKILLS) objectives and criteria to [audit](TASK) against [Develop](TASK) an [audit](TASK) plan describing the [frameworks](SKILLS) standards methodology procedures and auditing tests [Review](TASK) target of evaluation [security objectives](SKILLS) and requirements based on the risk profile [Audit](TASK) compliance with [cybersecurity](SKILLS)-related applicable [laws](SKILLS) and regulations [Audit](TASK) conformity with [cybersecurity](SKILLS)-related applicable standards Execute the [audit](TASK) plan and collect evidence and measurements [Maintain](TASK) and [protect](TASK) the integrity of [audit](TASK) records [Develop](TASK) and [communicate](TASK) [conformity assessment](SKILLS) assurance [audit](TASK) certification and [maintenance reports](SKILLS) [Monitor](TASK) [risk remediation activities](SKILLS)</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t xml:space="preserve"> [Organise](TASK) and [work](TASK) in a systematic and deterministic way based on evidence 
- [Follow](TASK) and [practice](TASK) auditing [frameworks](SKILLS), standards and [methodologies](SKILLS) 
- [Apply](TASK) [auditing tools](SKILLS) and techniques 
- [Analyse](TASK) business processes, [assess](TASK) and [review](TASK) software or hardware security, as  well as technical and organisational [controls](SKILLS) 
- [Decompose](TASK) and [analyse](TASK) [systems](SKILLS) to [identify](TASK) weaknesses and [ineffective controls](SKILLS) 
- [Communicate](TASK), [explain](TASK) and [adapt](TASK) legal and regulatory requirements and business needs 
- [Collect](TASK), [evaluate](TASK), [maintain](TASK) and [protect](TASK) auditing information 
- [Audit](TASK) with integrity, being impartial and independent
-</t>
+          <t>[Organise](TASK) and [work](TASK) in a systematic and deterministic way based on evidence [Follow](TASK) and [practice](TASK) auditing [frameworks](SKILLS) standards and [methodologies](SKILLS) [Apply](TASK) [auditing tools](SKILLS) and [techniques](TASK) [Analyse](TASK) business [processes](TASK) [assess](TASK) and [review](TASK) [software or hardware security](SKILLS) as well as technical and organisational [controls](SKILLS) [Decompose](TASK) and [analyse](TASK) [systems](SKILLS) to [identify](TASK) weaknesses and [ineffective controls](SKILLS) [Communicate](TASK) [explain](TASK) and [adapt](TASK) [legal](SKILLS) and regulatory requirements and business needs Collect [evaluate](TASK) [maintain](TASK) and [protect](TASK) auditing information [Audit](TASK) with integrity being impartial and independent</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>['Analyse', 'Apply', 'Audit', 'Collect', 'Communicate', 'Decompose', 'Define', 'Develop', 'Establish', 'Follow', 'Maintain', 'Monitor', 'Organise', 'Review', 'adapt', 'analyse', 'assess', 'audit', 'collect', 'communicate', 'evaluate', 'explain', 'identify', 'maintain', 'manage', 'practice', 'protect', 'review', 'work']</t>
+          <t>[Cybersecurity](SKILLS) [controls](SKILLS) and [solutions](SKILLS) [Legal regulatory](SKILLS) and legislative compliance requirements [recommendations](SKILLS) and [best practices](SKILLS) [Monitoring](SKILLS) [testing](TASK) and evaluating [cybersecurity](SKILLS) [controls](SKILLS)' effectiveness [Conformity assessment](SKILLS) [standards methodologies](SKILLS) and [frameworks](SKILLS) [Auditing standards](SKILLS) [methodologies](SKILLS) and [frameworks](SKILLS) [Cybersecurity standards methodologies](SKILLS) and [frameworks](SKILLS) Auditing-related certification [Cybersecurity](SKILLS)-related [certifications](SKILLS)</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>['audit scope', 'auditing policy', 'auditing tools', 'conformity assessment', 'controls', 'cybersecurity', 'frameworks', 'ineffective controls', 'maintenance reports', 'methodologies', 'products', 'regulatory frameworks', 'risk remediation activities', 'security objectives', 'services', 'systems', 'systems auditing']</t>
+          <t>['Analyse', 'Apply', 'Audit', 'Communicate', 'Decompose', 'Define', 'Develop', 'Establish', 'Evaluates', 'Follow', 'Maintain', 'Monitor', 'Organise', 'Review', 'adapt', 'analyse', 'assess', 'audit', 'communicate', 'evaluate', 'explain', 'identify', 'maintain', 'manage', 'practice', 'processes', 'protect', 'review', 'techniques', 'testing', 'work']</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>['Auditing standards', 'Conformity assessment', 'Cybersecurity', 'Cybersecurity standards methodologies', 'Legal regulatory', 'Monitoring', 'audit scope', 'auditing policy', 'auditing tools', 'best practices', 'certifications', 'conformity assessment', 'controls', 'cybersecurity', 'frameworks', 'ineffective controls', 'laws', 'legal', 'maintenance reports', 'methodologies', 'policies', 'products', 'recommendations', 'regulatory frameworks', 'risk remediation activities', 'security objectives', 'services', 'software or hardware security', 'solutions', 'standards methodologies', 'systems', 'systems auditing']</t>
         </is>
       </c>
     </row>
@@ -1143,7 +903,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Designs, develops and conducts awareness, training and educational programmes in  cybersecurity and data protection-related topics. Uses appropriate teaching and  training methods, techniques and instruments to communicate and enhance the  cybersecurity culture, capabilities, knowledge and skills of human resources.  Promotes the importance of cybersecurity and consolidates it into the organisation.</t>
+          <t>Designs develops and conducts awareness training and educational programmes in cybersecurity and data protection-related topics. Uses appropriate teaching and training methods techniques and instruments to communicate and enhance the cybersecurity culture capabilities knowledge and skills of human resources. Promotes the importance of cybersecurity and consolidates it into the organisation.</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1154,82 +914,47 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Develop, update and deliver cybersecurity and data protection curricula and  educational material for training and awareness based on content, method, tools,  trainees need 
- Organise, design and deliver cybersecurity and data protection awareness-raising  activities, seminars, courses, practical training 
- Monitor, evaluate and report training effectiveness 
- Evaluate and report trainee’s performance 
- Finding new approaches for education, training and awareness-raising 
- Design, develop and deliver cybersecurity simulations, virtual labs or cyber range  environments 
- Provide guidance on cybersecurity certification programs for individuals 
- Continuously maintain and enhance expertise; encourage and empower continuous  enhancement of cybersecurity capacities and capabilities building</t>
+          <t>Develop update and deliver cybersecurity and data protection curricula and educational material for training and awareness based on content method tools trainees need Organise design and deliver cybersecurity and data protection awareness-raising activities seminars courses practical training Monitor evaluate and report training effectiveness Evaluate and report trainee’s performance Finding new approaches for education training and awareness-raising Design develop and deliver cybersecurity simulations virtual labs or cyber range environments Provide guidance on cybersecurity certification programs for individuals Continuously maintain and enhance expertise; encourage and empower continuous enhancement of cybersecurity capacities and capabilities building</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Identify needs in cybersecurity awareness, training and education 
- Design, develop and deliver learning programmes to cover cybersecurity needs 
- Develop cybersecurity exercises including simulations using cyber range  environments 
- Provide training towards cybersecurity and data protection professional certifications 
- Utilise existing cybersecurity-related training resources 
- Develop evaluation programs for the awareness, training and education activities 
- Communicate, present and report to relevant stakeholders 
- Identify and select appropriate pedagogical approaches for the intended audience 
- Motivate and encourage people
-</t>
+          <t>Identify needs in cybersecurity awareness training and education Design develop and deliver learning programmes to cover cybersecurity needs Develop cybersecurity exercises including simulations using cyber range environments Provide training towards cybersecurity and data protection professional certifications Utilise existing cybersecurity-related training resources Develop evaluation programs for the awareness training and education activities Communicate present and report to relevant stakeholders Identify and select appropriate pedagogical approaches for the intended audience Motivate and encourage people</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Pedagogical standards, methodologies and frameworks 
- Cybersecurity awareness, education and training programme development 
- Cybersecurity-related certifications 
- Cybersecurity education and training standards, methodologies and frameworks 
- Cybersecurity related laws, regulations and legislations 
- Cybersecurity recommendations and best practices 
- Cybersecurity standards, methodologies and frameworks 
- Cybersecurity controls and solutions
-</t>
+          <t>Pedagogical standards methodologies and frameworks Cybersecurity awareness education and training programme development Cybersecurity-related certifications Cybersecurity education and training standards methodologies and frameworks Cybersecurity related laws regulations and legislations Cybersecurity recommendations and best practices Cybersecurity standards methodologies and frameworks Cybersecurity controls and solutions</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Designs, develops and conducts awareness, training and [educational programmes](SKILLS) in  [cybersecurity](SKILLS) and [data protection](SKILLS)-related topics. Uses appropriate teaching and  [training methods](SKILLS), techniques and instruments to [communicate](TASK) and [enhance](TASK) the  [cybersecurity](SKILLS) culture, capabilities, knowledge and skills of human resources.  Promotes the importance of [cybersecurity](SKILLS) and consolidates it into the organisation.</t>
+          <t>Designs develops and conducts [awareness training](SKILLS) and [educational programmes](SKILLS) in [cybersecurity](SKILLS) and [data protection](SKILLS)-related topics. Uses appropriate teaching and [training methods](SKILLS) [techniques](TASK) and instruments to [communicate](TASK) and [enhance](TASK) the [cybersecurity culture](SKILLS) capabilities knowledge and skills of human resources. Promotes the importance of [cybersecurity](SKILLS) and consolidates it into the organisation.</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t xml:space="preserve"> [Develop](TASK), [update](TASK) and [deliver](TASK) [cybersecurity](SKILLS) and [data protection](SKILLS) [curricula](SKILLS) and  educational material for training and awareness based on content, method, tools,  trainees need 
- [Organise](TASK), [design](TASK) and [deliver](TASK) [cybersecurity](SKILLS) and [data protection](SKILLS) awareness-raising  activities, seminars, courses, practical training 
- [Monitor](TASK), [evaluate](TASK) and [report](TASK) training effectiveness 
- [Evaluate](TASK) and [report](TASK) trainee’s performance 
- Finding new approaches for education, training and awareness-raising 
- [Design](TASK), [develop](TASK) and [deliver](TASK) [cybersecurity](SKILLS) simulations, [virtual labs](SKILLS) or cyber range  environments 
- [Provide](TASK) guidance on [cybersecurity](SKILLS) certification programs for individuals 
- Continuously [maintain](TASK) and [enhance](TASK) expertise; [encourage](TASK) and [empower](TASK) continuous  enhancement of [cybersecurity](SKILLS) capacities and capabilities building</t>
+          <t>[Develop](TASK) [update](TASK) and [deliver](TASK) [cybersecurity](SKILLS) and [data protection](SKILLS) curricula and educational material for [training](SKILLS) and awareness based on content method tools trainees need [Organise](TASK) [design](TASK) and [deliver](TASK) [cybersecurity](SKILLS) and [data protection](SKILLS) awareness-raising activities seminars courses practical [training](SKILLS) [Monitor](TASK) [evaluate](TASK) and [report](TASK) [training](SKILLS) effectiveness [Evaluate](TASK) and [report](TASK) trainee’s performance Finding new approaches for education [training](SKILLS) and awareness-raising [Design](TASK) [develop](TASK) and [deliver](TASK) [cybersecurity simulations](SKILLS) [virtual labs](SKILLS) or [cyber range environments](SKILLS) [Provide](TASK) guidance on [cybersecurity certification programs](SKILLS) for individuals Continuously [maintain](TASK) and [enhance](TASK) expertise; [encourage](TASK) and [empower](TASK) continuous enhancement of [cybersecurity](SKILLS) capacities and capabilities building</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t xml:space="preserve"> [Identify](TASK) needs in [cybersecurity](SKILLS) awareness, training and education 
- [Design](TASK), [develop](TASK) and [deliver](TASK) [learning programmes](SKILLS) to cover [cybersecurity](SKILLS) needs 
- [Develop](TASK) [cybersecurity](SKILLS) exercises including simulations using cyber range  environments 
- [Provide](TASK) training towards [cybersecurity](SKILLS) and [data protection](SKILLS) professional [certifications](SKILLS) 
- [Utilise](TASK) existing [cybersecurity](SKILLS)-related [training resources](SKILLS) 
- [Develop](TASK) [evaluation programs](SKILLS) for the awareness, training and education activities 
- [Communicate](TASK), [present](TASK) and [report](TASK) to relevant [stakeholders](SKILLS) 
- [Identify](TASK) and [select](TASK) appropriate [pedagogical approaches](SKILLS) for the intended audience 
- [Motivate](TASK) and [encourage](TASK) people
-</t>
+          <t>[Identify](TASK) needs in [cybersecurity awareness](SKILLS) [training](SKILLS) and education [Design](TASK) [develop](TASK) and [deliver](TASK) [learning programmes](SKILLS) to cover [cybersecurity](SKILLS) needs [Develop](TASK) [cybersecurity](SKILLS) exercises including simulations using [cyber range environments](SKILLS) [Provide](TASK) [training](SKILLS) towards [cybersecurity](SKILLS) and [data protection](SKILLS) professional [certifications](SKILLS) [Utilise](TASK) existing [cybersecurity](SKILLS)-related [training resources](SKILLS) [Develop](TASK) [evaluation programs](SKILLS) for the [awareness training](SKILLS) and education activities [Communicate](TASK) [present](TASK) and [report](TASK) to relevant stakeholders [Identify](TASK) and [select](TASK) appropriate [pedagogical approaches](SKILLS) for the intended audience [Motivate](TASK) and [encourage](TASK) people</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>['Communicate', 'Design', 'Develop', 'Evaluate', 'Identify', 'Monitor', 'Motivate', 'Organise', 'Provide', 'Utilise', 'communicate', 'deliver', 'design', 'develop', 'empower', 'encourage', 'enhance', 'evaluate', 'maintain', 'present', 'report', 'select', 'update']</t>
+          <t>Pedagogical [standards methodologies](SKILLS) and [frameworks](SKILLS) [Cybersecurity awareness](SKILLS) education and [training](SKILLS) programme development [Cybersecurity](SKILLS)-related [certifications](SKILLS) [Cybersecurity](SKILLS) education and [training](SKILLS) [standards methodologies](SKILLS) and [frameworks](SKILLS) [Cybersecurity](SKILLS) related [laws regulations](SKILLS) and legislations [Cybersecurity](SKILLS) [recommendations](SKILLS) and [best practices](SKILLS) [Cybersecurity standards methodologies](SKILLS) and [frameworks](SKILLS) [Cybersecurity](SKILLS) [controls](SKILLS) and [solutions](SKILLS)</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>['certifications', 'curricula', 'cybersecurity', 'data protection', 'educational programmes', 'evaluation programs', 'learning programmes', 'pedagogical approaches', 'stakeholders', 'training methods', 'training resources', 'virtual labs']</t>
+          <t>['Communicate', 'Design', 'Develop', 'Evaluate', 'Identify', 'Monitor', 'Motivate', 'Organise', 'Provide', 'Utilise', 'communicate', 'deliver', 'design', 'develop', 'empower', 'encourage', 'enhance', 'evaluate', 'maintain', 'present', 'report', 'select', 'techniques', 'update']</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>['Cybersecurity', 'Cybersecurity awareness', 'Cybersecurity standards methodologies', 'awareness training', 'best practices', 'certifications', 'controls', 'cyber range environments', 'cybersecurity', 'cybersecurity awareness', 'cybersecurity certification programs', 'cybersecurity culture', 'cybersecurity simulations', 'data protection', 'educational programmes', 'evaluation programs', 'frameworks', 'laws regulations', 'learning programmes', 'pedagogical approaches', 'recommendations', 'solutions', 'standards methodologies', 'training', 'training methods', 'training resources', 'virtual labs']</t>
         </is>
       </c>
     </row>
@@ -1244,7 +969,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Provides cybersecurity-related technical development, integration, testing,  implementation, operation, maintenance, monitoring and support of cybersecurity  solutions. Ensures adherence to specifications and conformance requirements,  assures sound performance and resolves technical issues required in the  organisation’s cybersecurity-related solutions (systems, assets, software, controls and  services), infrastructures and products.</t>
+          <t>Provides cybersecurity-related technical development integration testing implementation operation maintenance monitoring and support of cybersecurity solutions. Ensures adherence to specifications and conformance requirements assures sound performance and resolves technical issues required in the organisation’s cybersecurity-related solutions (systems assets software controls and services) infrastructures and products.</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1254,85 +979,47 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Develop, implement, maintain, upgrade, test cybersecurity products 
- Provide cybersecurity-related support to users and customers 
- Integrate cybersecurity solutions and ensure their sound operation 
- Securely configure systems, services and products 
- Maintain and upgrade the security of systems, services and products 
- Implement cybersecurity procedures and controls 
- Monitor and assure the performance of the implemented cybersecurity controls 
- Document and report on the security of systems, services and products 
- Work close with the IT/OT personnel on cybersecurity-related actions 
- Implement, apply and manage patches to products to address technical  vulnerabilities</t>
+          <t>Develop implement maintain upgrade test cybersecurity products Provide cybersecurity-related support to users and customers Integrate cybersecurity solutions and ensure their sound operation Securely configure systems services and products Maintain and upgrade the security of systems services and products Implement cybersecurity procedures and controls Monitor and assure the performance of the implemented cybersecurity controls Document and report on the security of systems services and products Work close with the IT/OT personnel on cybersecurity-related actions Implement apply and manage patches to products to address technical vulnerabilities</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Communicate, present and report to relevant stakeholders 
- Integrate cybersecurity solutions to the organisation’s infrastructure 
- Configure solutions according to the organisation’s security policy 
- Assess the security and performance of solutions 
- Develop code, scripts and programmes 
- Identify and solve cybersecurity-related issues 
- Collaborate with other team members and colleagues
-</t>
+          <t>Communicate present and report to relevant stakeholders Integrate cybersecurity solutions to the organisation’s infrastructure Configure solutions according to the organisation’s security policy Assess the security and performance of solutions Develop code scripts and programmes Identify and solve cybersecurity-related issues Collaborate with other team members and colleagues</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Secure development lifecycle 
- Computer programming 
- Operating systems security 
- Computer networks security 
- Cybersecurity controls and solutions 
- Offensive and defensive security practices 
- Secure coding recommendations and best practices 
- Cybersecurity recommendations and best practices 
- Testing standards, methodologies and frameworks 
- Testing procedures 
- Cybersecurity-related technologies
-</t>
+          <t>Secure development lifecycle Computer programming Operating systems security Computer networks security Cybersecurity controls and solutions Offensive and defensive security practices Secure coding recommendations and best practices Cybersecurity recommendations and best practices Testing standards methodologies and frameworks Testing procedures Cybersecurity-related technologies</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Provides [cybersecurity](SKILLS)-related [technical development](SKILLS), [integration](SKILLS), [testing](SKILLS),  [implementation](SKILLS), [operation](SKILLS), maintenance, [monitoring](SKILLS) and [support[](TASK)](SKILLS) of [cybersecurity](SKILLS)  [solutions](SKILLS). Ensures adherence to specifications and conformance requirements,  assures sound performance and resolves [technical issues](SKILLS) required in the  organisation’s [cybersecurity](SKILLS)-related [solutions](SKILLS) ([systems](SKILLS), [assets](SKILLS), software, [controls](SKILLS) and  [services](SKILLS)), [infrastructures](SKILLS) and [products](SKILLS).</t>
+          <t>Provides [cybersecurity](SKILLS)-related [technical development](SKILLS) [integration](SKILLS) [testing](TASK) [implementation](SKILLS) operation maintenance [monitoring](SKILLS) and [support](TASK) of [cybersecurity](SKILLS) [solutions](SKILLS). Ensures adherence to specifications and conformance requirements assures sound performance and resolves [technical issues](SKILLS) required in the organisation’s [cybersecurity](SKILLS)-related [solutions](SKILLS) ([systems](SKILLS) assets [software controls](SKILLS) and [services](SKILLS)) infrastructures and [products](SKILLS).</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t xml:space="preserve"> [Develop](TASK), [implement](TASK), [maintain](TASK), [upgrade](TASK), [test](TASK) [cybersecurity](SKILLS) [products](SKILLS) 
- [Provide](TASK) [cybersecurity](SKILLS)-related [support[](TASK)](SKILLS) to users and customers 
- [Integrate](TASK) [cybersecurity](SKILLS) [solutions](SKILLS) and [ensure](TASK) their sound [operation](SKILLS) 
- Securely [configure](TASK) [systems](SKILLS), [services](SKILLS) and [products](SKILLS) 
- [Maintain](TASK) and [upgrade](TASK) the security of [systems](SKILLS), [services](SKILLS) and [products](SKILLS) 
- [Implement](TASK) [cybersecurity](SKILLS) procedures and [controls](SKILLS) 
- [Monitor](TASK) and [assure](TASK) the performance of the implemented [cybersecurity](SKILLS) [controls](SKILLS) 
- [Document](TASK) and [report](TASK) on the security of [systems](SKILLS), [services](SKILLS) and [products](SKILLS) 
- [Work](TASK) close with the IT/OT personnel on [cybersecurity](SKILLS)-related actions 
- [Implement](TASK), [apply](TASK) and [manage](TASK) patches to [products](SKILLS) to address technical  vulnerabilities</t>
+          <t>[Develop](TASK) [implement](TASK) [maintain](TASK) [upgrade](TASK) [test](TASK) [cybersecurity](SKILLS) [products](SKILLS) [Provide](TASK) [cybersecurity](SKILLS)-related [support](TASK) to users and customers [Integrate](TASK) [cybersecurity](SKILLS) [solutions](SKILLS) and [ensure](TASK) their sound operation Securely [configure](TASK) [systems](SKILLS) [services](SKILLS) and [products](SKILLS) [Maintain](TASK) and [upgrade](TASK) the [security](SKILLS) of [systems](SKILLS) [services](SKILLS) and [products](SKILLS) [Implement](TASK) [cybersecurity](SKILLS) procedures and [controls](SKILLS) [Monitor](TASK) and [assure](TASK) the performance of the [implemented](TASK) [cybersecurity](SKILLS) [controls](SKILLS) [Document](TASK) and [report](TASK) on the [security](SKILLS) of [systems](SKILLS) [services](SKILLS) and [products](SKILLS) [Work](TASK) close with the IT/OT personnel on [cybersecurity](SKILLS)-related actions [Implement](TASK) [apply](TASK) and [manage](TASK) patches to [products](SKILLS) to address [technical vulnerabilities](SKILLS)</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t xml:space="preserve"> [Communicate](TASK), [present](TASK) and [report](TASK) to relevant [stakeholders](SKILLS) 
- [Integrate](TASK) [cybersecurity](SKILLS) [solutions](SKILLS) to the organisation’s infrastructure 
- [Configure](TASK) [solutions](SKILLS) according to the organisation’s security policy 
- [Assess](TASK) the security and performance of [solutions](SKILLS) 
- [Develop](TASK) code, scripts and programmes 
- [Identify](TASK) and [solve](TASK) [cybersecurity](SKILLS)-related issues 
- [Collaborate](TASK) with other team members and [colleagues](SKILLS)
-</t>
+          <t>[Communicate](TASK) [present](TASK) and [report](TASK) to relevant stakeholders [Integrate](TASK) [cybersecurity](SKILLS) [solutions](SKILLS) to the organisation’s infrastructure [Configure](TASK) [solutions](SKILLS) according to the organisation’s [security policy](SKILLS) [Assess](TASK) the [security](SKILLS) and performance of [solutions](SKILLS) [Develop](TASK) code scripts and programmes [Identify](TASK) and [solve](TASK) [cybersecurity-related issues](SKILLS) [Collaborate](TASK) with other team members and colleagues</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>['Assess', 'Collaborate', 'Communicate', 'Configure', 'Develop', 'Document', 'Identify', 'Implement', 'Integrate', 'Maintain', 'Monitor', 'Provide', 'Work', 'apply', 'assure', 'configure', 'ensure', 'implement', 'maintain', 'manage', 'present', 'report', 'solve', 'support', 'test', 'upgrade']</t>
+          <t>[Secure][(TASK) development](SKILLS) lifecycle Computer [programming](TASK) [Operating systems](SKILLS) [security](SKILLS) Computer [networks security](SKILLS) [Cybersecurity](SKILLS) [controls](SKILLS) and [solutions](SKILLS) [Offensive and defensive](SKILLS) [security](SKILLS) practices [Secure](TASK) coding [recommendations](SKILLS) and [best practices](SKILLS) [Cybersecurity](SKILLS) [recommendations](SKILLS) and [best practices](SKILLS) [Testing](TASK) [standards methodologies](SKILLS) and [frameworks](SKILLS) [Testing](TASK) procedures [Cybersecurity-related technologies](SKILLS)</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>['assets', 'colleagues', 'controls', 'cybersecurity', 'implementation', 'infrastructures', 'integration', 'monitoring', 'operation', 'products', 'services', 'solutions', 'stakeholders', 'support', 'systems', 'technical development', 'technical issues', 'testing']</t>
+          <t>['Assess', 'Collaborate', 'Communicate', 'Configure', 'Develop', 'Document', 'Identify', 'Implement', 'Integrate', 'Maintain', 'Monitor', 'Provide', 'Secure', 'Testing', 'Work', 'apply', 'assure', 'configure', 'ensure', 'implement', 'implemented', 'maintain', 'manage', 'present', 'programming', 'report', 'solve', 'support', 'test', 'testing', 'upgrade']</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>['Cybersecurity', 'Cybersecurity-related technologies', 'Offensive and defensive', 'Operating systems', 'Secure development', 'best practices', 'controls', 'cybersecurity', 'cybersecurity-related issues', 'frameworks', 'implementation', 'integration', 'monitoring', 'networks security', 'products', 'recommendations', 'security', 'security policy', 'services', 'software controls', 'solutions', 'standards methodologies', 'systems', 'technical development', 'technical issues', 'technical vulnerabilities']</t>
         </is>
       </c>
     </row>
@@ -1347,7 +1034,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Conducts fundamental/basic and applied research and facilitates innovation in the  cybersecurity domain through cooperation with other stakeholders. Analyses trends  and scientific findings in cybersecurity.</t>
+          <t>Conducts fundamental/basic and applied research and facilitates innovation in the cybersecurity domain through cooperation with other stakeholders. Analyses trends and scientific findings in cybersecurity.</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1357,81 +1044,47 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Analyse and assess cybersecurity technologies, solutions, developments and  processes 
- Conduct research, innovation and development work in cybersecurity-related topics
- Manifest and generate research and innovation ideas 
- Advance the current state-of-the-art in cybersecurity-related topics 
- Assist in the development of innovative cybersecurity-related solutions 
- Conduct experiments and develop a proof of concept, pilots and prototypes for  cybersecurity solutions 
- Select and apply frameworks, methods, standards, tools and protocols including a  building and testing a proof of concept to support projects 
- Contributes towards cutting-edge cybersecurity business ideas, services and  solutions 
- Assist in cybersecurity-related capacity building including awareness, theoretical  training, practical training, testing, mentoring, supervising and sharing  Identify cross-sectoral cybersecurity achievements and apply them in a different  context or propose innovative approaches and solutions 
- Lead or participate in the innovation processes and projects including project  management and budgeting 
- Publish and present scientific works and research and development results</t>
+          <t>Analyse and assess cybersecurity technologies solutions developments and processes Conduct research innovation and development work in cybersecurity-related topics Manifest and generate research and innovation ideas Advance the current state-of-the-art in cybersecurity-related topics Assist in the development of innovative cybersecurity-related solutions Conduct experiments and develop a proof of concept pilots and prototypes for cybersecurity solutions Select and apply frameworks methods standards tools and protocols including a building and testing a proof of concept to support projects Contributes towards cutting-edge cybersecurity business ideas services and solutions Assist in cybersecurity-related capacity building including awareness theoretical training practical training testing mentoring supervising and sharing Identify cross-sectoral cybersecurity achievements and apply them in a different context or propose innovative approaches and solutions Lead or participate in the innovation processes and projects including project management and budgeting Publish and present scientific works and research and development results</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Generate new ideas and transfer theory into practice 
- Decompose and analyse systems to identify weaknesses and ineffective controls 
- Decompose and analyse systems to develop security and privacy requirements and  identify effective solutions 
- Monitor new advancements in cybersecurity-related technologies 
- Communicate, present and report to relevant stakeholders 
- Identify and solve cybersecurity-related issues 
- Collaborate with other team members and colleagues
-</t>
+          <t>Generate new ideas and transfer theory into practice Decompose and analyse systems to identify weaknesses and ineffective controls Decompose and analyse systems to develop security and privacy requirements and identify effective solutions Monitor new advancements in cybersecurity-related technologies Communicate present and report to relevant stakeholders Identify and solve cybersecurity-related issues Collaborate with other team members and colleagues</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Cybersecurity-related research, development and innovation (RDI) 
- Cybersecurity standards, methodologies and frameworks 
- Legal, regulatory and legislative requirements on releasing or using cybersecurity  related technologies 
- Multidiscipline aspect of cybersecurity 
- Responsible information disclosure procedures
-</t>
+          <t>Cybersecurity-related research development and innovation (RDI) Cybersecurity standards methodologies and frameworks Legal regulatory and legislative requirements on releasing or using cybersecurity related technologies Multidiscipline aspect of cybersecurity Responsible information disclosure procedures</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Conducts fundamental/basic and applied research and facilitates innovation in the  [cybersecurity](SKILLS) domain through cooperation with other [stakeholders](SKILLS). Analyses trends  and scientific findings in [cybersecurity](SKILLS).</t>
+          <t>Conducts [fundamental](SKILLS)/basic and applied research and facilitates innovation in the [cybersecurity](SKILLS) domain through cooperation with other stakeholders. [Analyses](TASK) trends and scientific findings in [cybersecurity](SKILLS).</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t xml:space="preserve"> [Analyse](TASK) and [assess](TASK) [cybersecurity](SKILLS) technologies, [solutions](SKILLS), developments and  processes 
- [Conduct](TASK) research, innovation and development [work](TASK) in [cybersecurity](SKILLS)-related topics
- Manifest and generate research and innovation ideas 
- Advance the current state-of-the-art in [cybersecurity](SKILLS)-related topics 
- [Assist](TASK) in the development of innovative [cybersecurity](SKILLS)-related [solutions](SKILLS) 
- [Conduct](TASK) experiments and [develop](TASK) a proof of concept, pilots and prototypes for  [cybersecurity](SKILLS) [solutions](SKILLS) 
- [Select](TASK) and [apply](TASK) [frameworks](SKILLS), methods, standards, tools and protocols including a  building and [testing](SKILLS) a proof of concept to [support[](TASK)](SKILLS) projects 
- Contributes towards cutting-edge [cybersecurity](SKILLS) business ideas, [services](SKILLS) and  [solutions](SKILLS) 
- [Assist](TASK) in [cybersecurity](SKILLS)-related capacity building including awareness, theoretical  training, practical training, [testing](SKILLS), mentoring, supervising and sharing  [Identify](TASK) cross-sectoral [cybersecurity](SKILLS) achievements and [apply](TASK) them in a different  context or [propose](TASK) innovative approaches and [solutions](SKILLS) 
- [Lead](TASK) or participate in the innovation processes and projects including project  management and budgeting 
- Publish and [present](TASK) scientific works and research and development results</t>
+          <t>[Analyse](TASK) and [assess](TASK) [cybersecurity](SKILLS) technologies [solutions](SKILLS) developments and [processes](TASK) [Conduct](TASK) research innovation and development [work](TASK) in [cybersecurity](SKILLS)-related topics Manifest and generate research and innovation ideas Advance the current state-of-the-art in [cybersecurity](SKILLS)-related topics [Assist](TASK) in the development of innovative [cybersecurity](SKILLS)-related [solutions](SKILLS) [Conduct](TASK) experiments and [develop](TASK) a proof of concept pilots and prototypes for [cybersecurity](SKILLS) [solutions](SKILLS) [Select](TASK) and [apply](TASK) [frameworks](SKILLS) methods [standards tools and protocols](SKILLS) including a building and [testing](TASK) a proof of concept to [support](TASK) projects Contributes towards cutting-edge [cybersecurity](SKILLS) business ideas [services](SKILLS) and [solutions](SKILLS) [Assist](TASK) in [cybersecurity](SKILLS)-related capacity building including awareness theoretical [training](SKILLS) practical [training](SKILLS) [testing](TASK) mentoring supervising and sharing [Identify](TASK) cross-sectoral [cybersecurity](SKILLS) achievements and [apply](TASK) them in a different context or [propose](TASK) innovative approaches and [solutions](SKILLS) [Lead](TASK) or participate in the innovation [processes](TASK) and projects including project management and budgeting Publish and [present](TASK) scientific works and research and development results</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Generate new ideas and transfer theory into [practice](TASK) 
- [Decompose](TASK) and [analyse](TASK) [systems](SKILLS) to [identify](TASK) weaknesses and [ineffective controls](SKILLS) 
- [Decompose](TASK) and [analyse](TASK) [systems](SKILLS) to [develop](TASK) security and privacy requirements and  [identify](TASK) [effective solutions](SKILLS) 
- [Monitor](TASK) new advancements in [cybersecurity](SKILLS)-related technologies 
- [Communicate](TASK), [present](TASK) and [report](TASK) to relevant [stakeholders](SKILLS) 
- [Identify](TASK) and [solve](TASK) [cybersecurity](SKILLS)-related issues 
- [Collaborate](TASK) with other team members and [colleagues](SKILLS)
-</t>
+          <t>Generate new ideas and transfer theory into [practice](TASK) [Decompose](TASK) and [analyse](TASK) [systems](SKILLS) to [identify](TASK) weaknesses and [ineffective controls](SKILLS) [Decompose](TASK) and [analyse](TASK) [systems](SKILLS) to [develop](TASK) [security](SKILLS) and privacy requirements and [identify](TASK) [effective solutions](SKILLS) [Monitor](TASK) new advancements in [cybersecurity-related technologies](SKILLS) [Communicate](TASK) [present](TASK) and [report](TASK) to relevant stakeholders [Identify](TASK) and [solve](TASK) [cybersecurity-related issues](SKILLS) [Collaborate](TASK) with other team members and colleagues</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>['Analyse', 'Assist', 'Collaborate', 'Communicate', 'Conduct', 'Decompose', 'Identify', 'Lead', 'Monitor', 'Select', 'analyse', 'apply', 'assess', 'develop', 'identify', 'practice', 'present', 'propose', 'report', 'solve', 'support', 'work']</t>
+          <t>[Cybersecurity](SKILLS)-related research development and innovation (RDI) [Cybersecurity standards methodologies](SKILLS) and [frameworks](SKILLS) [Legal regulatory](SKILLS) and legislative requirements on releasing or using [cybersecurity](SKILLS) related technologies Multidiscipline aspect of [cybersecurity](SKILLS) Responsible information disclosure procedures</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>['colleagues', 'cybersecurity', 'effective solutions', 'frameworks', 'ineffective controls', 'services', 'solutions', 'stakeholders', 'support', 'systems', 'testing']</t>
+          <t>['Analyse', 'Analyses', 'Assist', 'Collaborate', 'Communicate', 'Conduct', 'Decompose', 'Identify', 'Lead', 'Monitor', 'Select', 'analyse', 'apply', 'assess', 'develop', 'identify', 'practice', 'present', 'processes', 'propose', 'report', 'solve', 'support', 'testing', 'work']</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>['Cybersecurity', 'Cybersecurity standards methodologies', 'Legal regulatory', 'cybersecurity', 'cybersecurity-related issues', 'cybersecurity-related technologies', 'effective solutions', 'frameworks', 'fundamental', 'ineffective controls', 'security', 'services', 'solutions', 'standards tools and protocols', 'systems', 'training']</t>
         </is>
       </c>
     </row>
@@ -1446,7 +1099,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Continuously manages (identifies, analyses, assesses, estimates, mitigates) the  cybersecurity-related risks of ICT infrastructures, systems and services by planning,  applying, reporting and communicating risk analysis, assessment and treatment.  Establishes a risk management strategy for the organisation and ensures that risks  remain at an acceptable level for the organisation by selecting mitigation actions and  controls.</t>
+          <t>Continuously manages (identifies analyses assesses estimates mitigates) the cybersecurity-related risks of ICT infrastructures systems and services by planning applying reporting and communicating risk analysis assessment and treatment. Establishes a risk management strategy for the organisation and ensures that risks remain at an acceptable level for the organisation by selecting mitigation actions and controls.</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1458,77 +1111,47 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Develop an organisation’s cybersecurity risk management strategy 
- Manage an inventory of organisation’s assets 
- Identify and assess cybersecurity-related threats and vulnerabilities of ICT systems 
- Identification of threat landscape including attackers’ profiles and estimation of  attacks’ potential 
- Assess cybersecurity risks and propose most appropriate risk treatment options,  including security controls and risk mitigation and avoidance that best address the  organisation’s strategy 
- Monitor effectiveness of cybersecurity controls and risk levels 
- Ensure that all cybersecurity risks remain at an acceptable level for the  organisation’s assets 
- Develop, maintain, report and communicate complete risk management cycle</t>
+          <t>Develop an organisation’s cybersecurity risk management strategy Manage an inventory of organisation’s assets Identify and assess cybersecurity-related threats and vulnerabilities of ICT systems Identification of threat landscape including attackers’ profiles and estimation of attacks’ potential Assess cybersecurity risks and propose most appropriate risk treatment options including security controls and risk mitigation and avoidance that best address the organisation’s strategy Monitor effectiveness of cybersecurity controls and risk levels Ensure that all cybersecurity risks remain at an acceptable level for the organisation’s assets Develop maintain report and communicate complete risk management cycle</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Implement cybersecurity risk management frameworks, methodologies and  guidelines and ensure compliance with regulations and standards 
- Analyse and consolidate organisation’s quality and risk management practices 
- Enable business assets owners, executives and other stakeholders to make risk informed decisions to manage and mitigate risks 
- Build a cybersecurity risk-aware environment 
- Communicate, present and report to relevant stakeholders 
- Propose and manage risk-sharing options
-</t>
+          <t>Implement cybersecurity risk management frameworks methodologies and guidelines and ensure compliance with regulations and standards Analyse and consolidate organisation’s quality and risk management practices Enable business assets owners executives and other stakeholders to make risk informed decisions to manage and mitigate risks Build a cybersecurity risk-aware environment Communicate present and report to relevant stakeholders Propose and manage risk-sharing options</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Risk management standards, methodologies and frameworks 
- Risk management tools 
- Risk management recommendations and best practices 
- Cyber threats 
- Computer systems vulnerabilities 
- Cybersecurity controls and solutions 
- Cybersecurity risks 
- Monitoring, testing and evaluating cybersecurity controls' effectiveness 
- Cybersecurity-related certifications 
- Cybersecurity-related technologies</t>
+          <t>Risk management standards methodologies and frameworks Risk management tools Risk management recommendations and best practices Cyber threats Computer systems vulnerabilities Cybersecurity controls and solutions Cybersecurity risks Monitoring testing and evaluating cybersecurity controls' effectiveness Cybersecurity-related certifications Cybersecurity-related technologies</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Continuously manages (identifies, analyses, assesses, estimates, mitigates) the  [cybersecurity](SKILLS)-related risks of ICT [infrastructures](SKILLS), [systems](SKILLS) and [services](SKILLS) by planning,  applying, reporting and communicating [risk analysis](SKILLS), assessment and treatment.  Establishes a [risk management](SKILLS) strategy for the organisation and ensures that risks  remain at an acceptable level for the organisation by selecting mitigation actions and  [controls](SKILLS).</t>
+          <t>Continuously [manages](TASK) (identifies [analyses](TASK) assesses estimates mitigates) the [cybersecurity](SKILLS)-related risks of ICT infrastructures [systems](SKILLS) and [services](SKILLS) by planning applying reporting and communicating [risk analysis](SKILLS) assessment and treatment. Establishes a [risk management](SKILLS) [strategy](SKILLS) for the organisation and ensures that risks remain at an acceptable level for the organisation by selecting mitigation actions and [controls](SKILLS).</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t xml:space="preserve"> [Develop](TASK) an organisation’s [cybersecurity](SKILLS) [risk management](SKILLS) strategy 
- [Manage](TASK) an inventory of organisation’s [assets](SKILLS) 
- [Identify](TASK) and [assess](TASK) [cybersecurity](SKILLS)-related threats and vulnerabilities of ICT [systems](SKILLS) 
- Identification of [threat landscape](SKILLS) including attackers’ profiles and estimation of  attacks’ potential 
- [Assess](TASK) [cybersecurity](SKILLS) risks and [propose](TASK) most appropriate [risk treatment options](SKILLS),  including [security controls](SKILLS) and [risk mitigation](SKILLS) and avoidance that best address the  organisation’s strategy 
- [Monitor](TASK) effectiveness of [cybersecurity](SKILLS) [controls](SKILLS) and risk levels 
- [Ensure](TASK) that all [cybersecurity](SKILLS) risks remain at an acceptable level for the  organisation’s [assets](SKILLS) 
- [Develop](TASK), [maintain](TASK), [report](TASK) and [communicate](TASK) complete [risk management](SKILLS) cycle</t>
+          <t>[Develop](TASK) an organisation’s [cybersecurity](SKILLS) [risk management](SKILLS) [strategy](SKILLS) [Manage](TASK) an inventory of organisation’s assets [Identify](TASK) and [assess](TASK) [cybersecurity](SKILLS)-related threats and [vulnerabilities](SKILLS) of ICT [systems](SKILLS) Identification of [threat landscape](SKILLS) including attackers’ profiles and estimation of [attacks](TASK)’ potential [Assess](TASK) [cybersecurity risks](SKILLS) and [propose](TASK) most appropriate risk treatment options including [security controls](SKILLS) and risk mitigation and avoidance that best address the organisation’s [strategy](SKILLS) [Monitor](TASK) effectiveness of [cybersecurity](SKILLS) [controls](SKILLS) and risk levels [Ensure](TASK) that all [cybersecurity risks](SKILLS) remain at an acceptable level for the organisation’s assets [Develop](TASK) [maintain](TASK) [report](TASK) and [communicate](TASK) complete [risk management](SKILLS) cycle</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t xml:space="preserve"> [Implement](TASK) [cybersecurity](SKILLS) [risk management](SKILLS) [frameworks](SKILLS), [methodologies](SKILLS) and  guidelines and [ensure](TASK) compliance with regulations and standards 
- [Analyse](TASK) and consolidate organisation’s quality and [risk management](SKILLS) practices 
- Enable business [assets](SKILLS) owners, executives and other [stakeholders](SKILLS) to make risk informed decisions to [manage](TASK) and [mitigate](TASK) risks 
- [Build](TASK) a [cybersecurity](SKILLS) risk-aware environment 
- [Communicate](TASK), [present](TASK) and [report](TASK) to relevant [stakeholders](SKILLS) 
- [Propose](TASK) and [manage](TASK) [risk-sharing options](SKILLS)
-</t>
+          <t>[Implement](TASK) [cybersecurity](SKILLS) [risk management](SKILLS) [frameworks](SKILLS) [methodologies](SKILLS) and guidelines and [ensure](TASK) compliance with regulations and standards [Analyse](TASK) and consolidate organisation’s quality and [risk management](SKILLS) practices Enable business assets owners executives and other stakeholders to make risk informed decisions to [manage](TASK) and mitigate risks [Build](TASK) a [cybersecurity](SKILLS) risk-aware environment [Communicate](TASK) [present](TASK) and [report](TASK) to relevant stakeholders [Propose](TASK) and [manage](TASK) [risk-sharing options](SKILLS)</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>['Analyse', 'Assess', 'Build', 'Communicate', 'Develop', 'Ensure', 'Identify', 'Implement', 'Manage', 'Monitor', 'Propose', 'assess', 'communicate', 'ensure', 'maintain', 'manage', 'mitigate', 'present', 'propose', 'report']</t>
+          <t>[Risk management](SKILLS) [standards methodologies](SKILLS) and [frameworks](SKILLS) [Risk management](SKILLS) tools [Risk management](SKILLS) [recommendations](SKILLS) and [best practices](SKILLS) [Cyber threats](SKILLS) Computer [systems](SKILLS) [vulnerabilities](SKILLS) [Cybersecurity](SKILLS) [controls](SKILLS) and [solutions](SKILLS) [Cybersecurity risks](SKILLS) [Monitoring](SKILLS) [testing](TASK) and evaluating [cybersecurity](SKILLS) [controls](SKILLS)' effectiveness [Cybersecurity](SKILLS)-related [certifications](SKILLS) [Cybersecurity-related technologies](SKILLS)</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>['assets', 'controls', 'cybersecurity', 'frameworks', 'infrastructures', 'methodologies', 'risk analysis', 'risk management', 'risk mitigation', 'risk treatment options', 'risk-sharing options', 'security controls', 'services', 'stakeholders', 'systems', 'threat landscape']</t>
+          <t>['Analyse', 'Assess', 'Build', 'Communicate', 'Develop', 'Ensure', 'Identify', 'Implement', 'Manage', 'Monitor', 'Propose', 'analyses', 'assess', 'attacks', 'communicate', 'ensure', 'maintain', 'manage', 'manages', 'present', 'propose', 'report', 'testing']</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>['Cyber threats', 'Cybersecurity', 'Cybersecurity risks', 'Cybersecurity-related technologies', 'Monitoring', 'Risk management', 'best practices', 'certifications', 'controls', 'cybersecurity', 'cybersecurity risks', 'frameworks', 'methodologies', 'recommendations', 'risk analysis', 'risk management', 'risk-sharing options', 'security controls', 'services', 'solutions', 'standards methodologies', 'strategy', 'systems', 'threat landscape', 'vulnerabilities']</t>
         </is>
       </c>
     </row>
@@ -1543,7 +1166,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Connects artefacts to natural persons, captures, recovers, identifies and preserves  data, including manifestations, inputs, outputs and processes of digital systems under  investigation. Provides analysis, reconstruction and interpretation of the digital  evidence based on a qualitative opinion. Presents an unbiased qualitative view  without interpreting the resultant findings.</t>
+          <t>Connects artefacts to natural persons captures recovers identifies and preserves data including manifestations inputs outputs and processes of digital systems under investigation. Provides analysis reconstruction and interpretation of the digital evidence based on a qualitative opinion. Presents an unbiased qualitative view without interpreting the resultant findings.</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1555,75 +1178,47 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Develop digital forensics investigation policy, plans and procedures 
- Identify, recover, extract, document and analyse digital evidence 
- Preserve and protect digital evidence and make it available to authorised  stakeholders 
- Inspect environments for evidence of unauthorised and unlawful actions 
- Systematically and deterministic document, report and present digital forensic  analysis findings and results 
- Select and customise forensics testing, analysing and reporting techniques</t>
+          <t>Develop digital forensics investigation policy plans and procedures Identify recover extract document and analyse digital evidence Preserve and protect digital evidence and make it available to authorised stakeholders Inspect environments for evidence of unauthorised and unlawful actions Systematically and deterministic document report and present digital forensic analysis findings and results Select and customise forensics testing analysing and reporting techniques</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Work ethically and independently; not influenced and biased by internal or external  actors 
- Collect information while preserving its integrity 
- Identify, analyse and correlate cybersecurity events 
- Explain and present digital evidence in a simple, straightforward and easy to  understand way 
- Develop and communicate, detailed and reasoned investigation reports
-</t>
+          <t>Work ethically and independently; not influenced and biased by internal or external actors Collect information while preserving its integrity Identify analyse and correlate cybersecurity events Explain and present digital evidence in a simple straightforward and easy to understand way Develop and communicate detailed and reasoned investigation reports</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Digital forensics recommendations and best practices 
- Digital forensics standards, methodologies and frameworks 
- Digital forensics analysis procedures 
- Testing procedures 
- Criminal investigation procedures, standards, methodologies and frameworks 
- Cybersecurity related laws, regulations and legislations  
- Malware analysis tools 
- Cyber threats 
- Computer systems vulnerabilities 
- Cybersecurity attack procedures 
- Operating systems security 
- Computer networks security 
- Cybersecurity-related certifications
-</t>
+          <t>Digital forensics recommendations and best practices Digital forensics standards methodologies and frameworks Digital forensics analysis procedures Testing procedures Criminal investigation procedures standards methodologies and frameworks Cybersecurity related laws regulations and legislations Malware analysis tools Cyber threats Computer systems vulnerabilities Cybersecurity attack procedures Operating systems security Computer networks security Cybersecurity-related certifications</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Connects [artefacts](SKILLS) to natural persons, captures, recovers, identifies and preserves  data, including manifestations, inputs, outputs and processes of digital [systems](SKILLS) under  investigation. Provides analysis, reconstruction and interpretation of the digital  evidence based on a qualitative opinion. Presents an unbiased qualitative view  without interpreting the resultant findings.</t>
+          <t>Connects artefacts to natural persons captures recovers identifies and preserves [data](SKILLS) including manifestations inputs outputs and [processes](TASK) of digital [systems](SKILLS) under investigation. Provides analysis reconstruction and interpretation of the [digital evidence](SKILLS) based on a qualitative opinion. Presents an unbiased qualitative view without interpreting the resultant findings.</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t xml:space="preserve"> [Develop](TASK) digital forensics investigation policy, plans and procedures 
- [Identify](TASK), [recover](TASK), [extract](TASK), [document](TASK) and [analyse](TASK) [digital evidence](SKILLS) 
- [Preserve](TASK) and [protect](TASK) [digital evidence](SKILLS) and make it available to authorised  [stakeholders](SKILLS) 
- [Inspect](TASK) environments for evidence of unauthorised and unlawful actions 
- Systematically and deterministic [document](TASK), [report](TASK) and [present](TASK) digital forensic  analysis findings and results 
- [Select](TASK) and [customise](TASK) forensics [testing](SKILLS), analysing and [reporting techniques](SKILLS)</t>
+          <t>[Develop](TASK) [digital forensics](SKILLS) investigation [policy](SKILLS) plans and procedures [Identify](TASK) [recover](TASK) [extract](TASK) [document](TASK) and [analyse](TASK) [digital evidence](SKILLS) [Preserve](TASK) and [protect](TASK) [digital evidence](SKILLS) and make it available to authorised stakeholders Inspect environments for evidence of unauthorised and unlawful actions Systematically and deterministic [document](TASK) [report](TASK) and [present](TASK) digital [forensic analysis](SKILLS) findings and results [Select](TASK) and [customise](TASK) forensics [testing](TASK) analysing and [reporting technique[s](SKILLS)](TASK)</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t xml:space="preserve"> [Work](TASK) ethically and independently; not influenced and biased by internal or external  actors 
- [Collect](TASK) information while preserving its integrity 
- [Identify](TASK), [analyse](TASK) and [correlate](TASK) [cybersecurity](SKILLS) events 
- [Explain](TASK) and [present](TASK) [digital evidence](SKILLS) in a simple, straightforward and easy to  understand way 
- [Develop](TASK) and [communicate](TASK), detailed and reasoned [investigation reports](SKILLS)
-</t>
+          <t>[Work](TASK) ethically and independently; not influenced and biased by internal or external actors Collect information while preserving its integrity [Identify](TASK) [analyse](TASK) and [correlate](TASK) [cybersecurity events](SKILLS) [Explain](TASK) and [present](TASK) [digital evidence](SKILLS) in a simple straightforward and easy to understand way [Develop](TASK) and [communicate](TASK) detailed and reasoned [investigation reports](SKILLS)</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>['Collect', 'Develop', 'Explain', 'Identify', 'Inspect', 'Preserve', 'Select', 'Work', 'analyse', 'communicate', 'correlate', 'customise', 'document', 'extract', 'present', 'protect', 'recover', 'report']</t>
+          <t>[Digital forensics](SKILLS) [recommendations](SKILLS) and [best practices](SKILLS) [Digital forensics](SKILLS) [standards methodologies](SKILLS) and [frameworks](SKILLS) [Digital forensics](SKILLS) analysis procedures [Testing](TASK) procedures Criminal investigation procedures [standards methodologies](SKILLS) and [frameworks](SKILLS) [Cybersecurity](SKILLS) related [laws regulations](SKILLS) and legislations [Malware analysis](SKILLS) tools [Cyber threats](SKILLS) Computer [systems](SKILLS) [vulnerabilities](SKILLS) [Cybersecurity attack pr[ocedur](TASK)es](SKILLS) [Operating systems](SKILLS) [security](SKILLS) Computer [networks security](SKILLS) [Cybersecurity](SKILLS)-related [certifications](SKILLS)</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>['artefacts', 'cybersecurity', 'digital evidence', 'investigation reports', 'reporting techniques', 'stakeholders', 'systems', 'testing']</t>
+          <t>['Develop', 'Explain', 'Identify', 'Preserve', 'Select', 'Testing', 'Work', 'analyse', 'attack', 'communicate', 'correlate', 'customise', 'document', 'extract', 'present', 'processes', 'protect', 'recover', 'report', 'techniques', 'testing']</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>['Cyber threats', 'Cybersecurity', 'Cybersecurity attack procedures', 'Digital forensics', 'Malware analysis', 'Operating systems', 'best practices', 'certifications', 'cybersecurity events', 'data', 'digital evidence', 'digital forensics', 'forensic analysis', 'frameworks', 'investigation reports', 'laws regulations', 'networks security', 'policy', 'recommendations', 'reporting techniques', 'security', 'standards methodologies', 'systems', 'vulnerabilities']</t>
         </is>
       </c>
     </row>
@@ -1638,7 +1233,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Plans, designs, implements and executes penetration testing activities and attack  scenarios to evaluate the effectiveness of deployed or planned security measures.  Identifies vulnerabilities or failures on technical and organisational controls that affect  the confidentiality, integrity and availability of ICT products (e.g. systems, hardware,  software and services).</t>
+          <t>Plans designs implements and executes penetration testing activities and attack scenarios to evaluate the effectiveness of deployed or planned security measures. Identifies vulnerabilities or failures on technical and organisational controls that affect the confidentiality integrity and availability of ICT products (e.g. systems hardware software and services).</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1650,88 +1245,47 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Identify, analyse and assess technical and organisational cybersecurity  vulnerabilities 
- Identify attack vectors, uncover and demonstrate exploitation of technical  cybersecurity vulnerabilities 
- Test systems and operations compliance with regulatory standards 
- Select and develop appropriate penetration testing techniques 
- Organise test plans and procedures for penetration testing 
- Establish procedures for penetration testing result analysis and reporting 
- Document and report penetration testing results to stakeholders 
- Deploy penetration testing tools and test programs</t>
+          <t>Identify analyse and assess technical and organisational cybersecurity vulnerabilities Identify attack vectors uncover and demonstrate exploitation of technical cybersecurity vulnerabilities Test systems and operations compliance with regulatory standards Select and develop appropriate penetration testing techniques Organise test plans and procedures for penetration testing Establish procedures for penetration testing result analysis and reporting Document and report penetration testing results to stakeholders Deploy penetration testing tools and test programs</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Develop codes, scripts and programmes 
- Perform social engineering 
- Identify and exploit vulnerabilities 
- Conduct ethical hacking 
- Think creatively and outside the box 
- Identify and solve cybersecurity-related issues 
- Communicate, present and report to relevant stakeholders 
- Use penetration testing tools effectively 
- Conduct technical analysis and reporting 
- Decompose and analyse systems to identify weaknesses and ineffective controls  Review codes assess their security
-</t>
+          <t>Develop codes scripts and programmes Perform social engineering Identify and exploit vulnerabilities Conduct ethical hacking Think creatively and outside the box Identify and solve cybersecurity-related issues Communicate present and report to relevant stakeholders Use penetration testing tools effectively Conduct technical analysis and reporting Decompose and analyse systems to identify weaknesses and ineffective controls Review codes assess their security</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Cybersecurity attack procedures 
- Information technology (IT) and operational technology (OT) appliances 
- Offensive and defensive security procedures 
- Operating systems security 
- Computer networks security 
- Penetration testing procedures 
- Penetration testing standards, methodologies and frameworks 
- Penetration testing tools 
- Computer programming 
- Computer systems vulnerabilities 
- Cybersecurity recommendations and best practices 
- Cybersecurity-related certifications
-</t>
+          <t>Cybersecurity attack procedures Information technology (IT) and operational technology (OT) appliances Offensive and defensive security procedures Operating systems security Computer networks security Penetration testing procedures Penetration testing standards methodologies and frameworks Penetration testing tools Computer programming Computer systems vulnerabilities Cybersecurity recommendations and best practices Cybersecurity-related certifications</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Plans, designs, implements and executes [penetration testing](SKILLS) activities and attack  scenarios to [evaluate](TASK) the effectiveness of deployed or planned [security measures](SKILLS).  Identifies vulnerabilities or failures on technical and organisational [controls](SKILLS) that affect  the confidentiality, integrity and availability of ICT [products](SKILLS) (e.g. [systems](SKILLS), hardware,  software and [services](SKILLS)).</t>
+          <t>Plans designs implements and executes [penetration testing]([SKILLS)](TASK) activities and [attack](TASK) scenarios to [evaluate](TASK) the effectiveness of deployed or planned [security measures](SKILLS). Identifies [vulnerabilities](SKILLS) or failures on technical and organisational [controls](SKILLS) that affect the confidentiality integrity and availability of ICT [products](SKILLS) (e.g. [systems](SKILLS) hardware software and [services](SKILLS)).</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t xml:space="preserve"> [Identify](TASK), [analyse](TASK) and [assess](TASK) technical and organisational [cybersecurity](SKILLS)  vulnerabilities 
- [Identify](TASK) [attack vectors](SKILLS), uncover and demonstrate exploitation of technical  [cybersecurity](SKILLS) vulnerabilities 
- [Test](TASK) [systems](SKILLS) and operations compliance with regulatory standards 
- [Select](TASK) and [develop](TASK) appropriate [penetration testing](SKILLS) techniques 
- [Organise](TASK) [test](TASK) plans and procedures for [penetration testing](SKILLS) 
- [Establish](TASK) procedures for [penetration testing](SKILLS) result analysis and reporting 
- [Document](TASK) and [report](TASK) [penetration testing](SKILLS) results to [stakeholders](SKILLS) 
- Deploy [penetration testing](SKILLS) tools and [test](TASK) programs</t>
+          <t>[Identify](TASK) [analyse](TASK) and [assess](TASK) technical and organisational [cybersecurity](SKILLS) [vulnerabilities](SKILLS) [Identify](TASK) [attack][(TASK) vectors](SKILLS) uncover and demonstrate exploitation of technical [cybersecurity](SKILLS) [vulnerabilities](SKILLS) [Test](TASK) [systems](SKILLS) and operations compliance with regulatory standards [Select](TASK) and [develop](TASK) appropriate [penetration testing]([SKILLS)](TASK) [techniques](TASK) [Organise test plans](TASK) and procedures for [penetration testing]([SKILLS)](TASK) [Establish](TASK) procedures for [penetration testing]([SKILLS)](TASK) result analysis and reporting [Document](TASK) and [report](TASK) [penetration testing]([SKILLS)](TASK) results to stakeholders Deploy [penetration testing]([SKILLS)](TASK) tools and [test](TASK) programs</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t xml:space="preserve"> [Develop](TASK) codes, scripts and programmes 
- [Perform social [engineering](TASK)](SKILLS) 
- [Identify](TASK) and [exploit vulnerabilities](TASK) 
- [Conduct](TASK) [ethical hacking](SKILLS) 
- [Think creatively](TASK) and outside the box 
- [Identify](TASK) and [solve](TASK) [cybersecurity](SKILLS)-related issues 
- [Communicate](TASK), [present](TASK) and [report](TASK) to relevant [stakeholders](SKILLS) 
- [Use](TASK) [penetration testing](SKILLS) tools effectively 
- [Conduct](TASK) [technical analysis](SKILLS) and reporting 
- [Decompose](TASK) and [analyse](TASK) [systems](SKILLS) to [identify](TASK) weaknesses and [ineffective controls](SKILLS)  [Review](TASK) codes [assess](TASK) their security
-</t>
+          <t>[Develop](TASK) codes scripts and programmes [Perform social [engineering](TASK)](SKILLS) [Identify](TASK) and [exploit vulnera[bilities](TASK)](SKILLS) [Conduct ethical[ hacking](TASK)](SKILLS) [Think creatively](TASK) and outside the box [Identify](TASK) and [solve](TASK) [cybersecurity-related issues](SKILLS) [Communicate](TASK) [present](TASK) and [report](TASK) to relevant stakeholders [Use](TASK) [penetration testing]([SKILLS)](TASK) tools effectively [Conduct](TASK) [technical analysis](SKILLS) and reporting [Decompose](TASK) and [analyse](TASK) [systems](SKILLS) to [identify](TASK) weaknesses and [ineffective controls](SKILLS) [Review](TASK) codes [assess](TASK) their [security](SKILLS)</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>['Communicate', 'Conduct', 'Decompose', 'Develop', 'Document', 'Establish', 'Identify', 'Organise', 'Perform social engineering', 'Review', 'Select', 'Test', 'Think creatively', 'Use', 'analyse', 'assess', 'develop', 'evaluate', 'exploit vulnerabilities', 'identify', 'present', 'report', 'solve', 'test']</t>
+          <t>[Cybersecurity attack pr[ocedur](TASK)es](SKILLS) Information technology (IT) and [operational](SKILLS) technology (OT) appliances [Offensive and defensive](SKILLS) [security](SKILLS) procedures [Operating systems](SKILLS) [security](SKILLS) Computer [networks security](SKILLS) [Penetration testing]([SKILLS)](TASK) procedures [Penetration testing]([SKILLS)](TASK) [standards methodologies](SKILLS) and [frameworks](SKILLS) [Penetration testing]([SKILLS)](TASK) tools Computer [programming](TASK) Computer [systems](SKILLS) [vulnerabilities](SKILLS) [Cybersecurity](SKILLS) [recommendations](SKILLS) and [best practices](SKILLS) [Cybersecurity](SKILLS)-related [certifications](SKILLS)</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>['attack vectors', 'controls', 'cybersecurity', 'ethical hacking', 'ineffective controls', 'penetration testing', 'products', 'security measures', 'services', 'social engineering', 'stakeholders', 'systems', 'technical analysis']</t>
+          <t>['Communicate', 'Conduct', 'Conduct ethical hacking', 'Decompose', 'Develop', 'Document', 'Establish', 'Identify', 'Organise test plans', 'Perform social engineering', 'Review', 'Select', 'Test', 'Think creatively', 'Use', 'analyse', 'assess', 'attack', 'develop', 'evaluate', 'exploit vulnerabilities', 'identify', 'present', 'programming', 'report', 'solve', 'techniques', 'test', 'testing']</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>['Cybersecurity', 'Cybersecurity attack procedures', 'Offensive and defensive', 'Operating systems', 'Penetration testing', 'attack vectors', 'best practices', 'certifications', 'controls', 'cybersecurity', 'cybersecurity-related issues', 'ethical hacking', 'frameworks', 'ineffective controls', 'networks security', 'operational', 'penetration testing', 'products', 'recommendations', 'security', 'security measures', 'services', 'social engineering', 'standards methodologies', 'systems', 'technical analysis', 'vulnerabilities']</t>
         </is>
       </c>
     </row>

</xml_diff>